<commit_message>
Apply bounded PM corrections to fusion review
</commit_message>
<xml_diff>
--- a/research/structural-profiles-pilot/domain-review/fusion_domain_review_v1.xlsx
+++ b/research/structural-profiles-pilot/domain-review/fusion_domain_review_v1.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rec05b33e91d84d8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profile review" sheetId="2" r:id="R761fb5c128e94026"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimension review" sheetId="3" r:id="R5ef53dc192a0406b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Load-bearing gaps" sheetId="4" r:id="Rd49ab1a65d9846d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="5" r:id="R15906f1a4561494e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner exceptions" sheetId="6" r:id="R3a195672db484e1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human experts" sheetId="7" r:id="R7be2fb3a4f594b6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preserved record" sheetId="8" r:id="R8e8e188c17544a89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R660aa80e8f2b49a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R81ccdd0b49fb4c3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profile review" sheetId="2" r:id="R8390e675212c412c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimension review" sheetId="3" r:id="R39dc5f65d9304658"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Load-bearing gaps" sheetId="4" r:id="R437981973bf8474f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="5" r:id="Ra83ee0852cdb4c83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner exceptions" sheetId="6" r:id="Refcb79adddb740b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human experts" sheetId="7" r:id="Rfadfbc95efea4796"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach packages" sheetId="8" r:id="R0787220e1d7445b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preserved record" sheetId="9" r:id="R61c62e93d6e448b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R6ddf4b20b21e45dc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -164,10 +165,10 @@
     <x:xf numFmtId="200" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -288,7 +289,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="OwnerexceptionsTable" displayName="OwnerexceptionsTable" ref="A4:I31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="OwnerexceptionsTable" displayName="OwnerexceptionsTable" ref="A4:I32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Profile ID"/>
     <x:tableColumn id="2" name="Dimension"/>
@@ -305,23 +306,42 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="HumanexpertsTable" displayName="HumanexpertsTable" ref="A4:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="8">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="HumanexpertsTable" displayName="HumanexpertsTable" ref="A4:K23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
     <x:tableColumn id="1" name="Profile ID"/>
     <x:tableColumn id="2" name="Dimension"/>
-    <x:tableColumn id="3" name="Question for named specialist"/>
-    <x:tableColumn id="4" name="Why load-bearing"/>
-    <x:tableColumn id="5" name="Canonical source IDs"/>
-    <x:tableColumn id="6" name="Requested expertise"/>
-    <x:tableColumn id="7" name="Named reviewer"/>
-    <x:tableColumn id="8" name="Status"/>
+    <x:tableColumn id="3" name="Outreach package"/>
+    <x:tableColumn id="4" name="Question for named specialist"/>
+    <x:tableColumn id="5" name="Why load-bearing"/>
+    <x:tableColumn id="6" name="Canonical source IDs"/>
+    <x:tableColumn id="7" name="Requested expertise"/>
+    <x:tableColumn id="8" name="Blocking stage"/>
+    <x:tableColumn id="9" name="Draft-use status"/>
+    <x:tableColumn id="10" name="Named reviewer"/>
+    <x:tableColumn id="11" name="Status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="PreservedrecordTable" displayName="PreservedrecordTable" ref="A4:O94" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="OutreachpackagesTable" displayName="OutreachpackagesTable" ref="A4:H10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="Package ID"/>
+    <x:tableColumn id="2" name="Theme"/>
+    <x:tableColumn id="3" name="Cell-level questions"/>
+    <x:tableColumn id="4" name="Question count"/>
+    <x:tableColumn id="5" name="Primary expertise"/>
+    <x:tableColumn id="6" name="Blocking stage"/>
+    <x:tableColumn id="7" name="Draft-use status"/>
+    <x:tableColumn id="8" name="Purpose"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PreservedrecordTable" displayName="PreservedrecordTable" ref="A4:O94" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="Profile ID"/>
     <x:tableColumn id="2" name="Dimension"/>
@@ -343,8 +363,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="SourcesTable" displayName="SourcesTable" ref="A4:H34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="SourcesTable" displayName="SourcesTable" ref="A4:H34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Canonical source ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -620,7 +640,7 @@
       </x:c>
       <x:c r="B7" s="20" t="n">
         <x:f>COUNTIF('Dimension review'!J5:J94,"range")</x:f>
-        <x:v>33</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C7" s="3" t="str">
         <x:v>Includes ranges routed to experts, evidence gaps and variants.</x:v>
@@ -635,7 +655,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="C8" s="3" t="str">
-        <x:v>A targeted gate, not a claim that other cells are approved.</x:v>
+        <x:v>All 19 cell questions remain; specialist sign-off has not occurred.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="32" customHeight="1">
@@ -643,23 +663,30 @@
         <x:v>Owner exceptions</x:v>
       </x:c>
       <x:c r="B9" s="20" t="n">
-        <x:f>COUNTA('Owner exceptions'!A5:A31)</x:f>
-        <x:v>27</x:v>
+        <x:f>COUNTA('Owner exceptions'!A5:A32)</x:f>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C9" s="3" t="str">
         <x:v>Exception view only; no need to re-review all 90 cells.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="3"/>
-      <x:c r="B10" s="21"/>
-      <x:c r="C10" s="3"/>
+    <x:row r="10" ht="32" customHeight="1">
+      <x:c r="A10" s="3" t="str">
+        <x:v>Expert outreach packages</x:v>
+      </x:c>
+      <x:c r="B10" s="20" t="n">
+        <x:f>COUNTA('Outreach packages'!A5:A10)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C10" s="3" t="str">
+        <x:v>Six coordinated outreach requests cover all 19 cell questions.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="27" customHeight="1">
       <x:c r="A11" s="8" t="str">
         <x:v>Disposition (one per cell)</x:v>
       </x:c>
-      <x:c r="B11" s="22" t="str">
+      <x:c r="B11" s="21" t="str">
         <x:v>Count</x:v>
       </x:c>
       <x:c r="C11" s="8" t="str">
@@ -670,9 +697,9 @@
       <x:c r="A12" s="3" t="str">
         <x:v>supports_current_record</x:v>
       </x:c>
-      <x:c r="B12" s="21" t="n">
+      <x:c r="B12" s="22" t="n">
         <x:f>COUNTIF('Dimension review'!L5:L94,A12)</x:f>
-        <x:v>46</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C12" s="3" t="str">
         <x:v>Supports coder agreement or an owner preference; does not approve the cell.</x:v>
@@ -682,9 +709,9 @@
       <x:c r="A13" s="3" t="str">
         <x:v>recommends_value_change</x:v>
       </x:c>
-      <x:c r="B13" s="21" t="n">
+      <x:c r="B13" s="22" t="n">
         <x:f>COUNTIF('Dimension review'!L5:L94,A13)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C13" s="3" t="str">
         <x:v>Prefers one submitted mark over another; no production S value changed.</x:v>
@@ -694,9 +721,9 @@
       <x:c r="A14" s="3" t="str">
         <x:v>recommends_range</x:v>
       </x:c>
-      <x:c r="B14" s="21" t="n">
+      <x:c r="B14" s="22" t="n">
         <x:f>COUNTIF('Dimension review'!L5:L94,A14)</x:f>
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C14" s="3" t="str">
         <x:v>Routine dimension-specific range; no midpoint or weighted combination.</x:v>
@@ -706,9 +733,9 @@
       <x:c r="A15" s="3" t="str">
         <x:v>insufficient_evidence</x:v>
       </x:c>
-      <x:c r="B15" s="21" t="n">
+      <x:c r="B15" s="22" t="n">
         <x:f>COUNTIF('Dimension review'!L5:L94,A15)</x:f>
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C15" s="3" t="str">
         <x:v>Candidate value/range only; decisive empirical support remains missing.</x:v>
@@ -718,7 +745,7 @@
       <x:c r="A16" s="3" t="str">
         <x:v>requires_human_expert</x:v>
       </x:c>
-      <x:c r="B16" s="21" t="n">
+      <x:c r="B16" s="22" t="n">
         <x:f>COUNTIF('Dimension review'!L5:L94,A16)</x:f>
         <x:v>14</x:v>
       </x:c>
@@ -730,7 +757,7 @@
       <x:c r="A17" s="3" t="str">
         <x:v>requires_pathway_variant</x:v>
       </x:c>
-      <x:c r="B17" s="21" t="n">
+      <x:c r="B17" s="22" t="n">
         <x:f>COUNTIF('Dimension review'!L5:L94,A17)</x:f>
         <x:v>6</x:v>
       </x:c>
@@ -742,7 +769,7 @@
       <x:c r="A18" s="3" t="str">
         <x:v>requires_jurisdiction_variant</x:v>
       </x:c>
-      <x:c r="B18" s="21" t="n">
+      <x:c r="B18" s="22" t="n">
         <x:f>COUNTIF('Dimension review'!L5:L94,A18)</x:f>
         <x:v>2</x:v>
       </x:c>
@@ -752,14 +779,14 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="3"/>
-      <x:c r="B19" s="21"/>
+      <x:c r="B19" s="22"/>
       <x:c r="C19" s="3"/>
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
       <x:c r="A20" s="8" t="str">
         <x:v>Recommendation confidence</x:v>
       </x:c>
-      <x:c r="B20" s="22" t="str">
+      <x:c r="B20" s="21" t="str">
         <x:v>Count</x:v>
       </x:c>
       <x:c r="C20" s="8" t="str">
@@ -770,7 +797,7 @@
       <x:c r="A21" s="3" t="str">
         <x:v>high</x:v>
       </x:c>
-      <x:c r="B21" s="21" t="n">
+      <x:c r="B21" s="22" t="n">
         <x:f>COUNTIF('Dimension review'!K5:K94,A21)</x:f>
         <x:v>12</x:v>
       </x:c>
@@ -782,9 +809,9 @@
       <x:c r="A22" s="3" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="B22" s="21" t="n">
+      <x:c r="B22" s="22" t="n">
         <x:f>COUNTIF('Dimension review'!K5:K94,A22)</x:f>
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C22" s="3" t="str">
         <x:v>Defensible structural interpretation with bounded transfer limits.</x:v>
@@ -794,9 +821,9 @@
       <x:c r="A23" s="3" t="str">
         <x:v>low</x:v>
       </x:c>
-      <x:c r="B23" s="21" t="n">
+      <x:c r="B23" s="22" t="n">
         <x:f>COUNTIF('Dimension review'!K5:K94,A23)</x:f>
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C23" s="3" t="str">
         <x:v>Sparse/adjacent evidence, uncertain ordinary cycle or unverified assurance boundary.</x:v>
@@ -836,61 +863,65 @@
     </x:row>
     <x:row r="28" ht="61" customHeight="1">
       <x:c r="A28" s="19" t="str">
-        <x:v>Candidate numbers</x:v>
+        <x:v>PM correction</x:v>
       </x:c>
       <x:c r="B28" s="3" t="str">
-        <x:v>Ordinal qualitative recommendations for later adjudication, including provisional carry-forward intervals where evidence is insufficient. They are not measured rates, empirical uncertainty bounds or selected S values.</x:v>
+        <x:v>No P0 or structural failure. Accept 88 recommendations/routes unchanged as recommendation_only; correct only sp-0024/S2 and sp-0027/S2. This does not select canonical S values.</x:v>
       </x:c>
       <x:c r="C28" s="3"/>
     </x:row>
     <x:row r="29" ht="61" customHeight="1">
       <x:c r="A29" s="19" t="str">
-        <x:v>S5 boundary</x:v>
+        <x:v>Candidate numbers</x:v>
       </x:c>
       <x:c r="B29" s="3" t="str">
-        <x:v>Each S5 row names the assumed next independent assurance/control boundary. No source establishes a complete pilot assurance architecture. Do not count remote cascades or double-charge harms past an independent boundary.</x:v>
+        <x:v>Ordinal qualitative recommendations for later adjudication, including provisional carry-forward intervals where evidence is insufficient. They are not measured rates, empirical uncertainty bounds or selected S values.</x:v>
       </x:c>
       <x:c r="C29" s="3"/>
     </x:row>
     <x:row r="30" ht="61" customHeight="1">
       <x:c r="A30" s="19" t="str">
-        <x:v>No approval</x:v>
+        <x:v>S5 boundary</x:v>
       </x:c>
       <x:c r="B30" s="3" t="str">
-        <x:v>All recommendations remain recommendation_only. Named reviewers are missing. No canonical source, raw submission, owner decision, existing S5 backlog or production data is changed.</x:v>
+        <x:v>Each S5 row names the assumed next independent assurance/control boundary. No source establishes a complete pilot assurance architecture. Do not count remote cascades or double-charge harms past an independent boundary.</x:v>
       </x:c>
       <x:c r="C30" s="3"/>
     </x:row>
     <x:row r="31" ht="61" customHeight="1">
       <x:c r="A31" s="19" t="str">
-        <x:v>Next gate</x:v>
+        <x:v>No approval</x:v>
       </x:c>
       <x:c r="B31" s="3" t="str">
-        <x:v>One substantive PM review and one correction pass, then merge this package. Separate 19-row targeted S5 adjudication follows later; WP2 remains out of scope.</x:v>
+        <x:v>All recommendations remain recommendation_only. Named reviewers are missing. EXPERT-CODED · DRAFT use does not create approved/canonical status. Protected records are unchanged.</x:v>
       </x:c>
       <x:c r="C31" s="3"/>
     </x:row>
     <x:row r="32" ht="61" customHeight="1">
       <x:c r="A32" s="19" t="str">
-        <x:v>Navigation</x:v>
+        <x:v>Next gate</x:v>
       </x:c>
       <x:c r="B32" s="3" t="str">
-        <x:v>Start with Owner exceptions and Human experts. Profile review summarizes 18 rows; Dimension review contains all 90 detailed assessments. Preserved record retains original rationales. Sources retains use restrictions.</x:v>
+        <x:v>PM substantive review and the bounded correction pass are complete. Merge remains a separate decision. Targeted S5 adjudication follows only later; WP2 is not implemented here.</x:v>
       </x:c>
       <x:c r="C32" s="3"/>
     </x:row>
     <x:row r="33" ht="61" customHeight="1">
       <x:c r="A33" s="19" t="str">
+        <x:v>Navigation</x:v>
+      </x:c>
+      <x:c r="B33" s="3" t="str">
+        <x:v>Start with Owner exceptions, Human experts and Outreach packages. Profile review summarizes 18 rows; Dimension review contains all 90 details. Preserved record retains original rationales.</x:v>
+      </x:c>
+      <x:c r="C33" s="3"/>
+    </x:row>
+    <x:row r="34" ht="61" customHeight="1">
+      <x:c r="A34" s="19" t="str">
         <x:v>Excluded evidence</x:v>
       </x:c>
-      <x:c r="B33" s="3" t="str">
+      <x:c r="B34" s="3" t="str">
         <x:v>fusion-src-013 and fusion-src-015 remain excluded. No STEP current target wording is used as load-bearing evidence; its failed-refresh restriction survives. No translated quotation or legal interpretation is approved.</x:v>
       </x:c>
-      <x:c r="C33" s="3"/>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="3"/>
-      <x:c r="B34" s="3"/>
       <x:c r="C34" s="3"/>
     </x:row>
     <x:row r="35">
@@ -941,8 +972,875 @@
     <x:mergeCell ref="B31:C31"/>
     <x:mergeCell ref="B32:C32"/>
     <x:mergeCell ref="B33:C33"/>
+    <x:mergeCell ref="B34:C34"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="84" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="106" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="31" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="35" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="107" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="150" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="54" customHeight="1">
+      <x:c r="A1" s="5" t="str">
+        <x:v>Sources</x:v>
+      </x:c>
+      <x:c r="B1" s="5"/>
+      <x:c r="C1" s="5"/>
+      <x:c r="D1" s="5"/>
+      <x:c r="E1" s="5"/>
+      <x:c r="F1" s="5"/>
+      <x:c r="G1" s="5"/>
+      <x:c r="H1" s="5"/>
+    </x:row>
+    <x:row r="2" ht="43" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>AI-assisted · recommendation only. Details extend to the right.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="3"/>
+      <x:c r="B3" s="3"/>
+      <x:c r="C3" s="3"/>
+      <x:c r="D3" s="3"/>
+      <x:c r="E3" s="3"/>
+      <x:c r="F3" s="3"/>
+      <x:c r="G3" s="3"/>
+      <x:c r="H3" s="3"/>
+    </x:row>
+    <x:row r="4" ht="43" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>Canonical source ID</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>Title</x:v>
+      </x:c>
+      <x:c r="C4" s="8" t="str">
+        <x:v>Primary / publisher URL</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="str">
+        <x:v>Independent-validation status</x:v>
+      </x:c>
+      <x:c r="E4" s="8" t="str">
+        <x:v>Evidence basis (bank)</x:v>
+      </x:c>
+      <x:c r="F4" s="8" t="str">
+        <x:v>Last verified</x:v>
+      </x:c>
+      <x:c r="G4" s="8" t="str">
+        <x:v>Source limitation</x:v>
+      </x:c>
+      <x:c r="H4" s="8" t="str">
+        <x:v>Promotion use restrictions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="76" customHeight="1">
+      <x:c r="A5" s="9" t="str">
+        <x:v>fusion-src-004</x:v>
+      </x:c>
+      <x:c r="B5" s="9" t="str">
+        <x:v>Atomic Energy Law of the People's Republic of China</x:v>
+      </x:c>
+      <x:c r="C5" s="9" t="str">
+        <x:v>https://www.caea.gov.cn/n6760338/n6760344/n10763762/n10763767/c10704020/content.html</x:v>
+      </x:c>
+      <x:c r="D5" s="9" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="E5" s="9" t="str">
+        <x:v>observed legal/regulatory status</x:v>
+      </x:c>
+      <x:c r="F5" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G5" s="9" t="str">
+        <x:v>An enacted law establishes legal status and authority; it is not a completed fusion licensing case or evidence of review duration. Earlier draft numbering differed, and final Article 37 concerns disused radioactive-source recovery/disposal.</x:v>
+      </x:c>
+      <x:c r="H5" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. An enacted law establishes legal status and authority; it is not a completed fusion licensing case or evidence of review duration. Earlier draft numbering differed, and final Article 37 concerns disused radioactive-source recovery/disposal. Direct public quotation or load-bearing translated wording remains blocked until the stated native-language/specialist review is completed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="44" customHeight="1">
+      <x:c r="A6" s="3" t="str">
+        <x:v>fusion-src-007</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="str">
+        <x:v>High-fidelity data-driven dynamics model for reinforcement learning-based control in HL-3 tokamak</x:v>
+      </x:c>
+      <x:c r="C6" s="3" t="str">
+        <x:v>https://doi.org/10.1038/s42005-025-02302-y</x:v>
+      </x:c>
+      <x:c r="D6" s="3" t="str">
+        <x:v>independently_validated</x:v>
+      </x:c>
+      <x:c r="E6" s="3" t="str">
+        <x:v>observed experimental result</x:v>
+      </x:c>
+      <x:c r="F6" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G6" s="3" t="str">
+        <x:v>Research-device demonstration; no nuclear-safety case, plant reliability, or transfer to pilot conditions.</x:v>
+      </x:c>
+      <x:c r="H6" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Research-device demonstration; no nuclear-safety case, plant reliability, or transfer to pilot conditions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="44" customHeight="1">
+      <x:c r="A7" s="9" t="str">
+        <x:v>fusion-src-008</x:v>
+      </x:c>
+      <x:c r="B7" s="9" t="str">
+        <x:v>Interpretability analysis and real-time prediction of locked mode-induced disruptions in EAST</x:v>
+      </x:c>
+      <x:c r="C7" s="9" t="str">
+        <x:v>https://doi.org/10.1088/1361-6587/ade5c5</x:v>
+      </x:c>
+      <x:c r="D7" s="9" t="str">
+        <x:v>independently_validated</x:v>
+      </x:c>
+      <x:c r="E7" s="9" t="str">
+        <x:v>proof of concept</x:v>
+      </x:c>
+      <x:c r="F7" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G7" s="9" t="str">
+        <x:v>Prediction performance is not autonomous avoidance, safe termination, or pilot-plant error tolerance.</x:v>
+      </x:c>
+      <x:c r="H7" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Prediction performance is not autonomous avoidance, safe termination, or pilot-plant error tolerance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="44" customHeight="1">
+      <x:c r="A8" s="3" t="str">
+        <x:v>fusion-src-009</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="str">
+        <x:v>Automatic identification of tokamak plasma confinement states with multi-task learning neural network</x:v>
+      </x:c>
+      <x:c r="C8" s="3" t="str">
+        <x:v>https://doi.org/10.1088/1741-4326/ade3ed</x:v>
+      </x:c>
+      <x:c r="D8" s="3" t="str">
+        <x:v>independently_validated</x:v>
+      </x:c>
+      <x:c r="E8" s="3" t="str">
+        <x:v>proof of concept</x:v>
+      </x:c>
+      <x:c r="F8" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G8" s="3" t="str">
+        <x:v>Classification benchmark; not a closed-loop control or safety demonstration.</x:v>
+      </x:c>
+      <x:c r="H8" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Classification benchmark; not a closed-loop control or safety demonstration.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="156" customHeight="1">
+      <x:c r="A9" s="9" t="str">
+        <x:v>fusion-src-011</x:v>
+      </x:c>
+      <x:c r="B9" s="9" t="str">
+        <x:v>Chinese fusion device sustains plasma operation for over 1,000 seconds</x:v>
+      </x:c>
+      <x:c r="C9" s="9" t="str">
+        <x:v>https://www.sh.news.cn/20260410/696d097c4a6c41b9af5f654314252a04/c.html</x:v>
+      </x:c>
+      <x:c r="D9" s="9" t="str">
+        <x:v>not_independently_validated</x:v>
+      </x:c>
+      <x:c r="E9" s="9" t="str">
+        <x:v>observed facility milestone</x:v>
+      </x:c>
+      <x:c r="F9" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G9" s="9" t="str">
+        <x:v>Official media repeats company data and explicitly describes low-parameter operation; not independent experimental validation, net energy, or plant availability.</x:v>
+      </x:c>
+      <x:c r="H9" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Official media repeats company data and explicitly describes low-parameter operation; not independent experimental validation, net energy, or plant availability. Reviewed source identity does not supply independent validation; company/operator reports and repeated company data must not be used as independently observed empirical outcomes. Rejected use fusion-rej-009: HH70 is a small, non-DT research tokamak without a breeder blanket, turbine, integrated tritium plant, or commercial nuclear commissioning. Permitted limited use: Optimistic analogue for small research-device iteration only. Do not transfer elapsed time to a pilot plant. Rejected use fusion-rej-010: Pulse duration and energy-turnover metrics omit blanket life, tritium-plant availability, component replacement, turbine/grid systems, downtime, and capacity factor. Permitted limited use: Plasma/facility milestone with device, discharge, and metric definitions preserved. No evidence of plant availability is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="108" customHeight="1">
+      <x:c r="A10" s="3" t="str">
+        <x:v>fusion-src-012</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="str">
+        <x:v>HH70 achieves first plasma</x:v>
+      </x:c>
+      <x:c r="C10" s="3" t="str">
+        <x:v>https://energysingularity.cn/en/news/news-025.html</x:v>
+      </x:c>
+      <x:c r="D10" s="3" t="str">
+        <x:v>not_independently_validated</x:v>
+      </x:c>
+      <x:c r="E10" s="3" t="str">
+        <x:v>observed facility milestone</x:v>
+      </x:c>
+      <x:c r="F10" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G10" s="3" t="str">
+        <x:v>First-party milestone; small non-DT device without blanket, tritium plant, turbine, or commercial licensing.</x:v>
+      </x:c>
+      <x:c r="H10" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. First-party milestone; small non-DT device without blanket, tritium plant, turbine, or commercial licensing. Reviewed source identity does not supply independent validation; company/operator reports and repeated company data must not be used as independently observed empirical outcomes. Rejected use fusion-rej-009: HH70 is a small, non-DT research tokamak without a breeder blanket, turbine, integrated tritium plant, or commercial nuclear commissioning. Permitted limited use: Optimistic analogue for small research-device iteration only. Do not transfer elapsed time to a pilot plant.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="44" customHeight="1">
+      <x:c r="A11" s="9" t="str">
+        <x:v>fusion-src-014</x:v>
+      </x:c>
+      <x:c r="B11" s="9" t="str">
+        <x:v>Development and construction of magnet system for world's first full high temperature superconducting tokamak</x:v>
+      </x:c>
+      <x:c r="C11" s="9" t="str">
+        <x:v>https://doi.org/10.1016/j.supcon.2024.100137</x:v>
+      </x:c>
+      <x:c r="D11" s="9" t="str">
+        <x:v>independently_validated</x:v>
+      </x:c>
+      <x:c r="E11" s="9" t="str">
+        <x:v>proof of concept</x:v>
+      </x:c>
+      <x:c r="F11" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G11" s="9" t="str">
+        <x:v>Magnet engineering does not validate the 1,337-second AI causal claim or a fusion power plant.</x:v>
+      </x:c>
+      <x:c r="H11" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Magnet engineering does not validate the 1,337-second AI causal claim or a fusion power plant.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="44" customHeight="1">
+      <x:c r="A12" s="3" t="str">
+        <x:v>fusion-src-017</x:v>
+      </x:c>
+      <x:c r="B12" s="3" t="str">
+        <x:v>Magnetic control of tokamak plasmas through deep reinforcement learning</x:v>
+      </x:c>
+      <x:c r="C12" s="3" t="str">
+        <x:v>https://doi.org/10.1038/s41586-021-04301-9</x:v>
+      </x:c>
+      <x:c r="D12" s="3" t="str">
+        <x:v>independently_validated</x:v>
+      </x:c>
+      <x:c r="E12" s="3" t="str">
+        <x:v>observed experimental result</x:v>
+      </x:c>
+      <x:c r="F12" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G12" s="3" t="str">
+        <x:v>Research tokamak; does not establish pilot-plant transfer, safety, reliability, or reduced nuclear commissioning time.</x:v>
+      </x:c>
+      <x:c r="H12" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Research tokamak; does not establish pilot-plant transfer, safety, reliability, or reduced nuclear commissioning time.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="44" customHeight="1">
+      <x:c r="A13" s="9" t="str">
+        <x:v>fusion-src-018</x:v>
+      </x:c>
+      <x:c r="B13" s="9" t="str">
+        <x:v>Avoiding fusion plasma tearing instability with deep reinforcement learning</x:v>
+      </x:c>
+      <x:c r="C13" s="9" t="str">
+        <x:v>https://doi.org/10.1038/s41586-024-07024-9</x:v>
+      </x:c>
+      <x:c r="D13" s="9" t="str">
+        <x:v>independently_validated</x:v>
+      </x:c>
+      <x:c r="E13" s="9" t="str">
+        <x:v>observed experimental result</x:v>
+      </x:c>
+      <x:c r="F13" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G13" s="9" t="str">
+        <x:v>Early proof of concept on a research device; not universal disruption avoidance or a nuclear-safety system.</x:v>
+      </x:c>
+      <x:c r="H13" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Early proof of concept on a research device; not universal disruption avoidance or a nuclear-safety system.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="92" customHeight="1">
+      <x:c r="A14" s="3" t="str">
+        <x:v>fusion-src-019</x:v>
+      </x:c>
+      <x:c r="B14" s="3" t="str">
+        <x:v>Highest fusion performance without harmful edge energy bursts in tokamak</x:v>
+      </x:c>
+      <x:c r="C14" s="3" t="str">
+        <x:v>https://doi.org/10.1038/s41467-024-48415-w</x:v>
+      </x:c>
+      <x:c r="D14" s="3" t="str">
+        <x:v>independently_validated</x:v>
+      </x:c>
+      <x:c r="E14" s="3" t="str">
+        <x:v>observed experimental result</x:v>
+      </x:c>
+      <x:c r="F14" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G14" s="3" t="str">
+        <x:v>Device- and scenario-specific experiment; the pack's simplified 'up to 90%' line is not promoted without a metric-matched locator.</x:v>
+      </x:c>
+      <x:c r="H14" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Device- and scenario-specific experiment; the pack's simplified 'up to 90%' line is not promoted without a metric-matched locator. Rejected use fusion-rej-005: The paper reports several device- and metric-specific changes; the pack's compressed percentage omits the exact metric, denominator, device, and condition. Permitted limited use: Cite the peer-reviewed cross-device experiment qualitatively or extract a metric-specific value with a Results/figure locator. The source remains staged; only the simplified number is rejected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="44" customHeight="1">
+      <x:c r="A15" s="9" t="str">
+        <x:v>fusion-src-020</x:v>
+      </x:c>
+      <x:c r="B15" s="9" t="str">
+        <x:v>Disruption prediction for future tokamaks using parameter-based transfer learning</x:v>
+      </x:c>
+      <x:c r="C15" s="9" t="str">
+        <x:v>https://doi.org/10.1038/s42005-023-01296-9</x:v>
+      </x:c>
+      <x:c r="D15" s="9" t="str">
+        <x:v>independently_validated</x:v>
+      </x:c>
+      <x:c r="E15" s="9" t="str">
+        <x:v>proof of concept</x:v>
+      </x:c>
+      <x:c r="F15" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G15" s="9" t="str">
+        <x:v>Offline, small-target-domain proof of concept; not live transfer to a future pilot plant.</x:v>
+      </x:c>
+      <x:c r="H15" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Offline, small-target-domain proof of concept; not live transfer to a future pilot plant.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="44" customHeight="1">
+      <x:c r="A16" s="3" t="str">
+        <x:v>fusion-src-021</x:v>
+      </x:c>
+      <x:c r="B16" s="3" t="str">
+        <x:v>Multimodal super-resolution: discovering hidden physics and its application to fusion plasmas</x:v>
+      </x:c>
+      <x:c r="C16" s="3" t="str">
+        <x:v>https://doi.org/10.1038/s41467-025-63492-1</x:v>
+      </x:c>
+      <x:c r="D16" s="3" t="str">
+        <x:v>independently_validated</x:v>
+      </x:c>
+      <x:c r="E16" s="3" t="str">
+        <x:v>proof of concept</x:v>
+      </x:c>
+      <x:c r="F16" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G16" s="3" t="str">
+        <x:v>Retrospective/synthetic diagnostic reconstruction; not a qualified replacement for safety instrumentation.</x:v>
+      </x:c>
+      <x:c r="H16" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Retrospective/synthetic diagnostic reconstruction; not a qualified replacement for safety instrumentation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="44" customHeight="1">
+      <x:c r="A17" s="9" t="str">
+        <x:v>fusion-src-022</x:v>
+      </x:c>
+      <x:c r="B17" s="9" t="str">
+        <x:v>GS-DeepNet: mastering tokamak plasma equilibria with deep neural networks and the Grad–Shafranov equation</x:v>
+      </x:c>
+      <x:c r="C17" s="9" t="str">
+        <x:v>https://doi.org/10.1038/s41598-023-42991-5</x:v>
+      </x:c>
+      <x:c r="D17" s="9" t="str">
+        <x:v>independently_validated</x:v>
+      </x:c>
+      <x:c r="E17" s="9" t="str">
+        <x:v>proof of concept</x:v>
+      </x:c>
+      <x:c r="F17" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G17" s="9" t="str">
+        <x:v>Model benchmark; not a closed-loop or safety-qualified deployment.</x:v>
+      </x:c>
+      <x:c r="H17" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Model benchmark; not a closed-loop or safety-qualified deployment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="60" customHeight="1">
+      <x:c r="A18" s="3" t="str">
+        <x:v>fusion-src-023</x:v>
+      </x:c>
+      <x:c r="B18" s="3" t="str">
+        <x:v>Finding the shadows in a fusion system faster with AI</x:v>
+      </x:c>
+      <x:c r="C18" s="3" t="str">
+        <x:v>https://www.pppl.gov/news/2025/finding-shadows-fusion-system-faster-ai</x:v>
+      </x:c>
+      <x:c r="D18" s="3" t="str">
+        <x:v>independently_validated</x:v>
+      </x:c>
+      <x:c r="E18" s="3" t="str">
+        <x:v>proof of concept</x:v>
+      </x:c>
+      <x:c r="F18" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G18" s="3" t="str">
+        <x:v>The present method covers 15 tiles in a small part of SPARC's exhaust geometry and is tied to that design; it is not plant-level schedule acceleration, materials qualification, or a generic plasma-facing-component result.</x:v>
+      </x:c>
+      <x:c r="H18" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. The present method covers 15 tiles in a small part of SPARC's exhaust geometry and is tied to that design; it is not plant-level schedule acceleration, materials qualification, or a generic plasma-facing-component result.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="60" customHeight="1">
+      <x:c r="A19" s="9" t="str">
+        <x:v>fusion-src-024</x:v>
+      </x:c>
+      <x:c r="B19" s="9" t="str">
+        <x:v>PPPL launches STELLAR-AI platform to accelerate fusion energy research</x:v>
+      </x:c>
+      <x:c r="C19" s="9" t="str">
+        <x:v>https://www.pppl.gov/news/2026/pppl-launches-stellar-ai-platform-accelerate-fusion-energy-research</x:v>
+      </x:c>
+      <x:c r="D19" s="9" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="E19" s="9" t="str">
+        <x:v>programme announcement</x:v>
+      </x:c>
+      <x:c r="F19" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G19" s="9" t="str">
+        <x:v>Programme announcement and capability intent, not an observed AI-shortened research cycle; its 'NSTX-U this year' wording was superseded by a 2027 experiment target.</x:v>
+      </x:c>
+      <x:c r="H19" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Programme announcement and capability intent, not an observed AI-shortened research cycle; its 'NSTX-U this year' wording was superseded by a 2027 experiment target.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="92" customHeight="1">
+      <x:c r="A20" s="3" t="str">
+        <x:v>fusion-src-026</x:v>
+      </x:c>
+      <x:c r="B20" s="3" t="str">
+        <x:v>MPEX user research forum 2026</x:v>
+      </x:c>
+      <x:c r="C20" s="3" t="str">
+        <x:v>https://mpex.ornl.gov/murf-2026/</x:v>
+      </x:c>
+      <x:c r="D20" s="3" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="E20" s="3" t="str">
+        <x:v>programme announcement</x:v>
+      </x:c>
+      <x:c r="F20" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G20" s="3" t="str">
+        <x:v>MPEX does not itself supply a fusion-spectrum neutron field; intended capability is not an observed qualification programme.</x:v>
+      </x:c>
+      <x:c r="H20" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. MPEX does not itself supply a fusion-spectrum neutron field; intended capability is not an observed qualification programme. Rejected use fusion-rej-011: MPEX is a plasma-materials exposure facility under assembly; it can test already neutron-irradiated specimens but is not itself a fusion-spectrum neutron source. Permitted limited use: Official intended capability for reactor-edge plasma exposure. Do not call intended capability completed qualification.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="44" customHeight="1">
+      <x:c r="A21" s="9" t="str">
+        <x:v>fusion-src-027</x:v>
+      </x:c>
+      <x:c r="B21" s="9" t="str">
+        <x:v>AI-accelerated fusion materials test facility</x:v>
+      </x:c>
+      <x:c r="C21" s="9" t="str">
+        <x:v>https://www.ornl.gov/research-highlight/ai-accelerated-fusion-materials-test-facility</x:v>
+      </x:c>
+      <x:c r="D21" s="9" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="E21" s="9" t="str">
+        <x:v>programme announcement</x:v>
+      </x:c>
+      <x:c r="F21" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G21" s="9" t="str">
+        <x:v>Announced/developing capability, not demonstrated materials qualification or component-life acceleration.</x:v>
+      </x:c>
+      <x:c r="H21" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Announced/developing capability, not demonstrated materials qualification or component-life acceleration.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="44" customHeight="1">
+      <x:c r="A22" s="3" t="str">
+        <x:v>fusion-src-028</x:v>
+      </x:c>
+      <x:c r="B22" s="3" t="str">
+        <x:v>Fusion Science and Technology Roadmap</x:v>
+      </x:c>
+      <x:c r="C22" s="3" t="str">
+        <x:v>https://www.energy.gov/documents/fusion-science-and-technology-roadmap</x:v>
+      </x:c>
+      <x:c r="D22" s="3" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="E22" s="3" t="str">
+        <x:v>programme announcement</x:v>
+      </x:c>
+      <x:c r="F22" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G22" s="3" t="str">
+        <x:v>Official roadmap and targets, not observed reductions in materials, blanket, tritium, licensing, or construction time.</x:v>
+      </x:c>
+      <x:c r="H22" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Official roadmap and targets, not observed reductions in materials, blanket, tritium, licensing, or construction time.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="60" customHeight="1">
+      <x:c r="A23" s="9" t="str">
+        <x:v>fusion-src-029</x:v>
+      </x:c>
+      <x:c r="B23" s="9" t="str">
+        <x:v>DIII-D National Fusion Program completes facility upgrade</x:v>
+      </x:c>
+      <x:c r="C23" s="9" t="str">
+        <x:v>https://www.ga.com/diii-d-national-fusion-program-completes-facility-upgrade</x:v>
+      </x:c>
+      <x:c r="D23" s="9" t="str">
+        <x:v>not_independently_validated</x:v>
+      </x:c>
+      <x:c r="E23" s="9" t="str">
+        <x:v>observed facility milestone</x:v>
+      </x:c>
+      <x:c r="F23" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G23" s="9" t="str">
+        <x:v>Facility milestone, not an AI result or a directly comparable nuclear commissioning programme.</x:v>
+      </x:c>
+      <x:c r="H23" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Facility milestone, not an AI result or a directly comparable nuclear commissioning programme. Reviewed source identity does not supply independent validation; company/operator reports and repeated company data must not be used as independently observed empirical outcomes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="124" customHeight="1">
+      <x:c r="A24" s="3" t="str">
+        <x:v>fusion-src-031</x:v>
+      </x:c>
+      <x:c r="B24" s="3" t="str">
+        <x:v>SPARC technology page</x:v>
+      </x:c>
+      <x:c r="C24" s="3" t="str">
+        <x:v>https://www.cfs.energy/technology/</x:v>
+      </x:c>
+      <x:c r="D24" s="3" t="str">
+        <x:v>not_independently_validated</x:v>
+      </x:c>
+      <x:c r="E24" s="3" t="str">
+        <x:v>company target</x:v>
+      </x:c>
+      <x:c r="F24" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G24" s="3" t="str">
+        <x:v>Company target and living page; no observed Q&gt;1 result or grid connection.</x:v>
+      </x:c>
+      <x:c r="H24" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Company target and living page; no observed Q&gt;1 result or grid connection. Reviewed source identity does not supply independent validation; company/operator reports and repeated company data must not be used as independently observed empirical outcomes. Rejected use fusion-rej-013: Targets and programme announcements do not demonstrate net energy, electricity export, fuel self-sufficiency, availability, or grid connection. Permitted limited use: Target tracking with owner, date, pathway, and target status preserved. No target is typed as an observed result. Promotion freshness check 2026-09-01: CFS SPARC milestones still place construction in progress and first plasma/net energy in the future; no outcome approval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="108" customHeight="1">
+      <x:c r="A25" s="9" t="str">
+        <x:v>fusion-src-032</x:v>
+      </x:c>
+      <x:c r="B25" s="9" t="str">
+        <x:v>New best values at Wendelstein 7-X</x:v>
+      </x:c>
+      <x:c r="C25" s="9" t="str">
+        <x:v>https://www.ipp.mpg.de/5532474/w7x</x:v>
+      </x:c>
+      <x:c r="D25" s="9" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="E25" s="9" t="str">
+        <x:v>observed experimental result</x:v>
+      </x:c>
+      <x:c r="F25" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G25" s="9" t="str">
+        <x:v>Different discharges/metrics; neither is net energy, DT operation, plant availability, or blanket life.</x:v>
+      </x:c>
+      <x:c r="H25" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Different discharges/metrics; neither is net energy, DT operation, plant availability, or blanket life. Direct public quotation or load-bearing translated wording remains blocked until the stated native-language/specialist review is completed. Rejected use fusion-rej-010: Pulse duration and energy-turnover metrics omit blanket life, tritium-plant availability, component replacement, turbine/grid systems, downtime, and capacity factor. Permitted limited use: Plasma/facility milestone with device, discharge, and metric definitions preserved. No evidence of plant availability is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="44" customHeight="1">
+      <x:c r="A26" s="3" t="str">
+        <x:v>fusion-src-033</x:v>
+      </x:c>
+      <x:c r="B26" s="3" t="str">
+        <x:v>First plasma 23 October</x:v>
+      </x:c>
+      <x:c r="C26" s="3" t="str">
+        <x:v>https://www.jt60sa.org/wp/first-plasma-23-october/</x:v>
+      </x:c>
+      <x:c r="D26" s="3" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="E26" s="3" t="str">
+        <x:v>observed facility milestone</x:v>
+      </x:c>
+      <x:c r="F26" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G26" s="3" t="str">
+        <x:v>Low-power research commissioning milestone; not high-power operation, DT commissioning, or commercial reliability.</x:v>
+      </x:c>
+      <x:c r="H26" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Low-power research commissioning milestone; not high-power operation, DT commissioning, or commercial reliability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="44" customHeight="1">
+      <x:c r="A27" s="9" t="str">
+        <x:v>fusion-src-034</x:v>
+      </x:c>
+      <x:c r="B27" s="9" t="str">
+        <x:v>OP2 has started</x:v>
+      </x:c>
+      <x:c r="C27" s="9" t="str">
+        <x:v>https://www.jt60sa.org/wp/op2-has-started/</x:v>
+      </x:c>
+      <x:c r="D27" s="9" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="E27" s="9" t="str">
+        <x:v>official target</x:v>
+      </x:c>
+      <x:c r="F27" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G27" s="9" t="str">
+        <x:v>Mixed current facility milestone and future target; not proof that the experimental campaign or high-power commissioning is complete.</x:v>
+      </x:c>
+      <x:c r="H27" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Mixed current facility milestone and future target; not proof that the experimental campaign or high-power commissioning is complete.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="44" customHeight="1">
+      <x:c r="A28" s="3" t="str">
+        <x:v>fusion-src-036</x:v>
+      </x:c>
+      <x:c r="B28" s="3" t="str">
+        <x:v>ITER Machine Assembly Overview</x:v>
+      </x:c>
+      <x:c r="C28" s="3" t="str">
+        <x:v>https://www.iter.org/project/assembly-overview</x:v>
+      </x:c>
+      <x:c r="D28" s="3" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="E28" s="3" t="str">
+        <x:v>official target</x:v>
+      </x:c>
+      <x:c r="F28" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G28" s="3" t="str">
+        <x:v>Official baseline proposal, not observed completion; later phases add nuclear/tritium systems.</x:v>
+      </x:c>
+      <x:c r="H28" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Official baseline proposal, not observed completion; later phases add nuclear/tritium systems.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="44" customHeight="1">
+      <x:c r="A29" s="9" t="str">
+        <x:v>fusion-src-037</x:v>
+      </x:c>
+      <x:c r="B29" s="9" t="str">
+        <x:v>Millions of data points, one successful lift</x:v>
+      </x:c>
+      <x:c r="C29" s="9" t="str">
+        <x:v>https://www.iter.org/node/20687/millions-data-points-one-successful-lift</x:v>
+      </x:c>
+      <x:c r="D29" s="9" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="E29" s="9" t="str">
+        <x:v>observed facility milestone</x:v>
+      </x:c>
+      <x:c r="F29" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G29" s="9" t="str">
+        <x:v>Observed construction/facility milestone only; not an AI result, integrated chamber completion, commissioning, or plant completion.</x:v>
+      </x:c>
+      <x:c r="H29" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Observed construction/facility milestone only; not an AI result, integrated chamber completion, commissioning, or plant completion.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="44" customHeight="1">
+      <x:c r="A30" s="3" t="str">
+        <x:v>fusion-src-038</x:v>
+      </x:c>
+      <x:c r="B30" s="3" t="str">
+        <x:v>Tritium breeding</x:v>
+      </x:c>
+      <x:c r="C30" s="3" t="str">
+        <x:v>https://www.iter.org/machine/supporting-systems/tritium-breeding</x:v>
+      </x:c>
+      <x:c r="D30" s="3" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="E30" s="3" t="str">
+        <x:v>programme announcement</x:v>
+      </x:c>
+      <x:c r="F30" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G30" s="3" t="str">
+        <x:v>Future test programme; ITER is not a tritium-self-sufficient power plant and testing is not qualification of a commercial blanket.</x:v>
+      </x:c>
+      <x:c r="H30" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Future test programme; ITER is not a tritium-self-sufficient power plant and testing is not qualification of a commercial blanket.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="44" customHeight="1">
+      <x:c r="A31" s="9" t="str">
+        <x:v>fusion-src-039</x:v>
+      </x:c>
+      <x:c r="B31" s="9" t="str">
+        <x:v>Regulatory Framework for Fusion Machines; Proposed Rule</x:v>
+      </x:c>
+      <x:c r="C31" s="9" t="str">
+        <x:v>https://www.federalregister.gov/documents/2026/02/26/2026-03865/regulatory-framework-for-fusion-machines</x:v>
+      </x:c>
+      <x:c r="D31" s="9" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="E31" s="9" t="str">
+        <x:v>observed legal/regulatory status</x:v>
+      </x:c>
+      <x:c r="F31" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G31" s="9" t="str">
+        <x:v>Proposed rule and draft guidance, not a final rule, observed plant-licence review, or licence-review-duration dataset.</x:v>
+      </x:c>
+      <x:c r="H31" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Proposed rule and draft guidance, not a final rule, observed plant-licence review, or licence-review-duration dataset.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="76" customHeight="1">
+      <x:c r="A32" s="3" t="str">
+        <x:v>fusion-src-040</x:v>
+      </x:c>
+      <x:c r="B32" s="3" t="str">
+        <x:v>Fusion Machine Rulemaking Status</x:v>
+      </x:c>
+      <x:c r="C32" s="3" t="str">
+        <x:v>https://www.nrc.gov/materials/fusion/rulemaking-status</x:v>
+      </x:c>
+      <x:c r="D32" s="3" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="E32" s="3" t="str">
+        <x:v>observed legal/regulatory status</x:v>
+      </x:c>
+      <x:c r="F32" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G32" s="3" t="str">
+        <x:v>Current regulator status, not evidence of licence throughput, a completed plant application, or licence-review duration.</x:v>
+      </x:c>
+      <x:c r="H32" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Current regulator status, not evidence of licence throughput, a completed plant application, or licence-review duration. Promotion freshness check 2026-09-01: NRC status page still lists the February proposed rule and draft guidance; footer remains 2026-08-27. No final rule or completed licence case is inferred.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="60" customHeight="1">
+      <x:c r="A33" s="9" t="str">
+        <x:v>fusion-src-045</x:v>
+      </x:c>
+      <x:c r="B33" s="9" t="str">
+        <x:v>The IFMIF-DONES Irradiation Modules</x:v>
+      </x:c>
+      <x:c r="C33" s="9" t="str">
+        <x:v>https://doi.org/10.1088/1741-4326/add172</x:v>
+      </x:c>
+      <x:c r="D33" s="9" t="str">
+        <x:v>independently_validated</x:v>
+      </x:c>
+      <x:c r="E33" s="9" t="str">
+        <x:v>model or scenario estimate</x:v>
+      </x:c>
+      <x:c r="F33" s="9" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G33" s="9" t="str">
+        <x:v>IFMIF-DONES and its modules are under design/development; no completed or accepted qualification dataset exists. Spectrum/transmutation matching is material-dependent: Eurofer is tailored, while tungsten/copper conditions are not perfectly matched.</x:v>
+      </x:c>
+      <x:c r="H33" s="9" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. IFMIF-DONES and its modules are under design/development; no completed or accepted qualification dataset exists. Spectrum/transmutation matching is material-dependent: Eurofer is tailored, while tungsten/copper conditions are not perfectly matched.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="60" customHeight="1">
+      <x:c r="A34" s="3" t="str">
+        <x:v>fusion-src-046</x:v>
+      </x:c>
+      <x:c r="B34" s="3" t="str">
+        <x:v>IFMIF-DONES: Experimental strategy for fusion materials qualification</x:v>
+      </x:c>
+      <x:c r="C34" s="3" t="str">
+        <x:v>https://conferences.iaea.org/event/406/contributions/37622/</x:v>
+      </x:c>
+      <x:c r="D34" s="3" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="E34" s="3" t="str">
+        <x:v>official target</x:v>
+      </x:c>
+      <x:c r="F34" s="3" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="G34" s="3" t="str">
+        <x:v>The facility is under construction and the values are programme design targets, not observed irradiation campaigns or a completed accepted qualification dataset. Post-irradiation examination remains part of the qualification chain.</x:v>
+      </x:c>
+      <x:c r="H34" s="3" t="str">
+        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. The facility is under construction and the values are programme design targets, not observed irradiation campaigns or a completed accepted qualification dataset. Post-irradiation examination remains part of the qualification chain.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:D1"/>
+    <x:mergeCell ref="A2:D2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0600383297a24e2b"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -1658,9 +2556,9 @@
 Broaden the shared 1 to 1-2 rather than infer work composition from missing pilot data.</x:v>
       </x:c>
       <x:c r="F15" s="9" t="str">
-        <x:v>0-1 | low
-insufficient_evidence
-A slow 0-1 candidate remains uncalibrated. The separate integrated empirical gap stays open without defining every development revision.</x:v>
+        <x:v>1 | low
+supports_current_record
+Support both original coder values at 1 without treating the open integrated outcome as a prerequisite for each pre-integration learning loop.</x:v>
       </x:c>
       <x:c r="G15" s="9" t="str">
         <x:v>1 | low
@@ -1829,9 +2727,9 @@
 Both 0s match the frozen construction scope.</x:v>
       </x:c>
       <x:c r="F18" s="3" t="str">
-        <x:v>0-2 | low
-recommends_range
-The shared 0 overstates certainty about cadence; keep 0-2 pending a defined decision-relevant construction loop.</x:v>
+        <x:v>1 | medium
+recommends_value_change
+Recommend 1 over both preserved coder values at 0 because the repeated work-package loop, rather than total facility duration, is the V1 S2 unit.</x:v>
       </x:c>
       <x:c r="G18" s="3" t="str">
         <x:v>0 | medium
@@ -2102,7 +3000,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6467f9f795ee4f48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf707e40947c84971"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6700,7 +7598,7 @@
         <x:v>dr-sp-0024-s1-v1</x:v>
       </x:c>
     </x:row>
-    <x:row r="56" ht="76" customHeight="1">
+    <x:row r="56" ht="108" customHeight="1">
       <x:c r="A56" s="3" t="str">
         <x:v>sp-0024</x:v>
       </x:c>
@@ -6725,29 +7623,29 @@
         <x:v>missing</x:v>
       </x:c>
       <x:c r="H56" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I56" s="13" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J56" s="3" t="str">
         <x:f>IF(H56=I56,"value","range")</x:f>
-        <x:v>range</x:v>
+        <x:v>value</x:v>
       </x:c>
       <x:c r="K56" s="3" t="str">
         <x:v>low</x:v>
       </x:c>
       <x:c r="L56" s="3" t="str">
-        <x:v>insufficient_evidence</x:v>
+        <x:v>supports_current_record</x:v>
       </x:c>
       <x:c r="M56" s="3" t="str">
-        <x:v>A slow 0-1 candidate remains uncalibrated. The separate integrated empirical gap stays open without defining every development revision.</x:v>
+        <x:v>Support both original coder values at 1 without treating the open integrated outcome as a prerequisite for each pre-integration learning loop.</x:v>
       </x:c>
       <x:c r="N56" s="3" t="str">
         <x:v>fusion-src-038;fusion-src-028</x:v>
       </x:c>
       <x:c r="O56" s="3" t="str">
-        <x:v>Dated revisions and results for representative pre-integration processing/extraction tests, with the claimed test endpoint specified.</x:v>
+        <x:v>Revisit if reviewed representative tritium-capable subsystem revision records support a materially different ordinary loop.</x:v>
       </x:c>
       <x:c r="P56" s="3" t="str">
         <x:v>false</x:v>
@@ -6765,10 +7663,10 @@
         <x:v>programme announcement</x:v>
       </x:c>
       <x:c r="U56" s="3" t="str">
-        <x:v>The ordinary loop is subsystem/process revision, representative testing and evaluation within pre-integration development. No source times that loop. Requiring a fully self-sufficient plant cycle would import later integration; programme dates do not supply development feedback.</x:v>
+        <x:v>The frozen row covers pilot-relevant tritium/fuel-cycle design, engineering, testing and pre-integration. The missing integrated self-sufficient breeder, extraction, processing and inventory-closure outcome remains gap-04, but that later integrated outcome is outside the ordinary feedback loop of this pre-integration development stage. Representative tritium-capable subsystem revisions remain scarce and slow, supporting 1 as the most defensible bounded candidate rather than an observed duration.</x:v>
       </x:c>
       <x:c r="V56" s="3" t="str">
-        <x:v>Future TBM breeding work is adjacent to fuel-cycle development; it neither times representative pre-integration tests nor demonstrates self-sufficiency.</x:v>
+        <x:v>The programme sources identify relevant functions but do not observe the duration of a representative tritium-capable subsystem revision or demonstrate self-sufficiency.</x:v>
       </x:c>
       <x:c r="W56" s="3" t="str">
         <x:v>not_applicable</x:v>
@@ -7990,7 +8888,7 @@
         <x:v>dr-sp-0027-s1-v1</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" ht="60" customHeight="1">
+    <x:row r="71" ht="108" customHeight="1">
       <x:c r="A71" s="9" t="str">
         <x:v>sp-0027</x:v>
       </x:c>
@@ -8015,35 +8913,35 @@
         <x:v>missing</x:v>
       </x:c>
       <x:c r="H71" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I71" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J71" s="9" t="str">
         <x:f>IF(H71=I71,"value","range")</x:f>
-        <x:v>range</x:v>
+        <x:v>value</x:v>
       </x:c>
       <x:c r="K71" s="9" t="str">
-        <x:v>low</x:v>
+        <x:v>medium</x:v>
       </x:c>
       <x:c r="L71" s="9" t="str">
-        <x:v>recommends_range</x:v>
+        <x:v>recommends_value_change</x:v>
       </x:c>
       <x:c r="M71" s="9" t="str">
-        <x:v>The shared 0 overstates certainty about cadence; keep 0-2 pending a defined decision-relevant construction loop.</x:v>
+        <x:v>Recommend 1 over both preserved coder values at 0 because the repeated work-package loop, rather than total facility duration, is the V1 S2 unit.</x:v>
       </x:c>
       <x:c r="N71" s="9" t="str">
         <x:v>fusion-src-037;fusion-src-036</x:v>
       </x:c>
       <x:c r="O71" s="9" t="str">
-        <x:v>A dated assembly/rework sequence distinguishing work-package feedback from total facility completion.</x:v>
+        <x:v>Revisit if a different construction learning unit is frozen, or if reviewed work-package/module cycle data support a materially different ordinary loop.</x:v>
       </x:c>
       <x:c r="P71" s="9" t="str">
         <x:v>false</x:v>
       </x:c>
       <x:c r="Q71" s="9" t="str">
-        <x:v>false</x:v>
+        <x:v>true</x:v>
       </x:c>
       <x:c r="R71" s="9" t="str">
         <x:v>Construction</x:v>
@@ -8055,10 +8953,10 @@
         <x:v>observed facility milestone; official target</x:v>
       </x:c>
       <x:c r="U71" s="9" t="str">
-        <x:v>A whole facility may take years, while fitting, inspecting and revising an assembly work package can close a shorter ordinary loop. Neither a full baseline schedule nor one successful lift identifies the representative learning unit.</x:v>
+        <x:v>S2 measures the ordinary learn-test-revise cycle inside the frozen stage, not the total duration of constructing the whole facility. For V1, use a repeatable major assembly/work-package loop: assemble, fit, inspect, diagnose deviations, revise procedures or tooling, and apply lessons to the next comparable package. That loop is months to roughly a year-plus, supporting the intermediate months-to-years value 1 rather than a range spanning years or decades through weeks or months.</x:v>
       </x:c>
       <x:c r="V71" s="9" t="str">
-        <x:v>ITER milestones establish staged construction, not a measured distribution of correction-cycle durations. HH70 build time is not a pilot-plant floor.</x:v>
+        <x:v>The retained canonical records show the construction sequence but do not calibrate an ordinary work-package cycle. PM external cross-checking of official ITER cycle records supports the months-scale judgment; those records are not canonical here and are not added to source IDs.</x:v>
       </x:c>
       <x:c r="W71" s="9" t="str">
         <x:v>not_applicable</x:v>
@@ -10067,7 +10965,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07a2df19b838471f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95d9885d8d124114"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10319,7 +11217,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R272d993aeaec4fb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f1577532aa2466f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10582,7 +11480,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re686feb0cd384969"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37b54836ea764ece"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11190,128 +12088,128 @@
         <x:v>fusion-src-014;fusion-src-037</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="76" customHeight="1">
+    <x:row r="23" ht="44" customHeight="1">
       <x:c r="A23" s="9" t="str">
+        <x:v>sp-0027</x:v>
+      </x:c>
+      <x:c r="B23" s="9" t="str">
+        <x:v>S2</x:v>
+      </x:c>
+      <x:c r="C23" s="9" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D23" s="9" t="str">
+        <x:v>recommends_value_change</x:v>
+      </x:c>
+      <x:c r="E23" s="9" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="F23" s="9" t="str">
+        <x:v>No owner decision recorded.</x:v>
+      </x:c>
+      <x:c r="G23" s="9" t="str">
+        <x:v>Revisit if a different construction learning unit is frozen, or if reviewed work-package/module cycle data support a materially different ordinary loop.</x:v>
+      </x:c>
+      <x:c r="H23" s="9" t="str">
+        <x:v>Recommend 1 over both preserved coder values at 0 because the repeated work-package loop, rather than total facility duration, is the V1 S2 unit.</x:v>
+      </x:c>
+      <x:c r="I23" s="9" t="str">
+        <x:v>fusion-src-037;fusion-src-036</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="76" customHeight="1">
+      <x:c r="A24" s="3" t="str">
         <x:v>sp-0028</x:v>
       </x:c>
-      <x:c r="B23" s="9" t="str">
+      <x:c r="B24" s="3" t="str">
         <x:v>S5</x:v>
       </x:c>
-      <x:c r="C23" s="9" t="str">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D23" s="9" t="str">
-        <x:v>requires_human_expert</x:v>
-      </x:c>
-      <x:c r="E23" s="9" t="str">
-        <x:v>prefer_seed</x:v>
-      </x:c>
-      <x:c r="F23" s="9" t="str">
-        <x:v>Select S5=1. Commissioning mistakes can damage unique installed hardware and create serious hazards, yet commissioning is deliberately staged, interlocked and reversible where practicable. The stage is low-tolerance, but S5=0 treats the severe tail as the ordinary error consequence.</x:v>
-      </x:c>
-      <x:c r="G23" s="9" t="str">
-        <x:v>During pilot nuclear/tritium commissioning, what direct harm from an erroneous startup or interface check can occur before independently verified interlocks and readiness hold points act?</x:v>
-      </x:c>
-      <x:c r="H23" s="9" t="str">
-        <x:v>Support owner 1 provisionally; obtain named expertise before canonical/public approval of this boundary.</x:v>
-      </x:c>
-      <x:c r="I23" s="9" t="str">
-        <x:v>fusion-src-033;fusion-src-034;fusion-src-036</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="44" customHeight="1">
-      <x:c r="A24" s="3" t="str">
-        <x:v>sp-0029</x:v>
-      </x:c>
-      <x:c r="B24" s="3" t="str">
-        <x:v>S2</x:v>
-      </x:c>
       <x:c r="C24" s="3" t="str">
-        <x:v>0-1</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D24" s="3" t="str">
         <x:v>requires_human_expert</x:v>
       </x:c>
       <x:c r="E24" s="3" t="str">
-        <x:v>missing</x:v>
+        <x:v>prefer_seed</x:v>
       </x:c>
       <x:c r="F24" s="3" t="str">
-        <x:v>No owner decision recorded.</x:v>
+        <x:v>Select S5=1. Commissioning mistakes can damage unique installed hardware and create serious hazards, yet commissioning is deliberately staged, interlocked and reversible where practicable. The stage is low-tolerance, but S5=0 treats the severe tail as the ordinary error consequence.</x:v>
       </x:c>
       <x:c r="G24" s="3" t="str">
-        <x:v>What specific pilot reliability or availability claim, exposure requirement and failure/repair criterion defines completion, and what ordinary learn-demonstrate-revise interval follows?</x:v>
+        <x:v>During pilot nuclear/tritium commissioning, what direct harm from an erroneous startup or interface check can occur before independently verified interlocks and readiness hold points act?</x:v>
       </x:c>
       <x:c r="H24" s="3" t="str">
-        <x:v>Keep a slow 0-1 candidate interval but do not assume the shared 0 proves a years-long statistical target.</x:v>
+        <x:v>Support owner 1 provisionally; obtain named expertise before canonical/public approval of this boundary.</x:v>
       </x:c>
       <x:c r="I24" s="3" t="str">
-        <x:v>fusion-src-011;fusion-src-032</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="76" customHeight="1">
+        <x:v>fusion-src-033;fusion-src-034;fusion-src-036</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="44" customHeight="1">
       <x:c r="A25" s="9" t="str">
         <x:v>sp-0029</x:v>
       </x:c>
       <x:c r="B25" s="9" t="str">
-        <x:v>S5</x:v>
+        <x:v>S2</x:v>
       </x:c>
       <x:c r="C25" s="9" t="str">
-        <x:v>1</x:v>
+        <x:v>0-1</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
         <x:v>requires_human_expert</x:v>
       </x:c>
       <x:c r="E25" s="9" t="str">
-        <x:v>prefer_seed</x:v>
+        <x:v>missing</x:v>
       </x:c>
       <x:c r="F25" s="9" t="str">
-        <x:v>Select S5=1. Component failures are the phenomenon reliability demonstration is designed to reveal and should not automatically be treated as errors by the stage. Errors in test conduct or inference can still waste irreplaceable operating time, so the stage remains low-tolerance rather than catastrophic by definition.</x:v>
+        <x:v>No owner decision recorded.</x:v>
       </x:c>
       <x:c r="G25" s="9" t="str">
-        <x:v>Which errors in reliability-test conduct or inference can escape to cause harm before independent machine protection and readiness acceptance, distinct from component failures the test is meant to reveal?</x:v>
+        <x:v>What specific pilot reliability or availability claim, exposure requirement and failure/repair criterion defines completion, and what ordinary learn-demonstrate-revise interval follows?</x:v>
       </x:c>
       <x:c r="H25" s="9" t="str">
-        <x:v>Support owner 1 provisionally with an explicit distinction between informative failure and erroneous assurance.</x:v>
+        <x:v>Keep a slow 0-1 candidate interval but do not assume the shared 0 proves a years-long statistical target.</x:v>
       </x:c>
       <x:c r="I25" s="9" t="str">
-        <x:v>missing</x:v>
+        <x:v>fusion-src-011;fusion-src-032</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="76" customHeight="1">
       <x:c r="A26" s="3" t="str">
-        <x:v>sp-0030</x:v>
+        <x:v>sp-0029</x:v>
       </x:c>
       <x:c r="B26" s="3" t="str">
-        <x:v>S2</x:v>
+        <x:v>S5</x:v>
       </x:c>
       <x:c r="C26" s="3" t="str">
-        <x:v>0-1</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D26" s="3" t="str">
-        <x:v>requires_jurisdiction_variant</x:v>
+        <x:v>requires_human_expert</x:v>
       </x:c>
       <x:c r="E26" s="3" t="str">
-        <x:v>needs_domain_review</x:v>
+        <x:v>prefer_seed</x:v>
       </x:c>
       <x:c r="F26" s="3" t="str">
-        <x:v>Do not select 0 or 1 yet. Licensing feedback speed is jurisdiction- and pathway-dependent, and the frozen row names no jurisdiction. A fusion-regulatory reviewer should determine whether a shared profile is defensible or whether U.S., Chinese and other licensing variants are required.</x:v>
+        <x:v>Select S5=1. Component failures are the phenomenon reliability demonstration is designed to reveal and should not automatically be treated as errors by the stage. Errors in test conduct or inference can still waste irreplaceable operating time, so the stage remains low-tolerance rather than catastrophic by definition.</x:v>
       </x:c>
       <x:c r="G26" s="3" t="str">
-        <x:v>Which jurisdiction-specific application, review and response stages define the ordinary fusion pilot licensing loop, and is any shared 0-1 recommendation defensible without a completed comparable case?</x:v>
+        <x:v>Which errors in reliability-test conduct or inference can escape to cause harm before independent machine protection and readiness acceptance, distinct from component failures the test is meant to reveal?</x:v>
       </x:c>
       <x:c r="H26" s="3" t="str">
-        <x:v>Carry 0-1 as an unadjudicated candidate range, not an empirical bound; do not select either owner-withheld value without a jurisdiction.</x:v>
+        <x:v>Support owner 1 provisionally with an explicit distinction between informative failure and erroneous assurance.</x:v>
       </x:c>
       <x:c r="I26" s="3" t="str">
-        <x:v>fusion-src-039;fusion-src-040;fusion-src-004</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="60" customHeight="1">
+        <x:v>missing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="76" customHeight="1">
       <x:c r="A27" s="9" t="str">
         <x:v>sp-0030</x:v>
       </x:c>
       <x:c r="B27" s="9" t="str">
-        <x:v>S3</x:v>
+        <x:v>S2</x:v>
       </x:c>
       <x:c r="C27" s="9" t="str">
         <x:v>0-1</x:v>
@@ -11323,74 +12221,74 @@
         <x:v>needs_domain_review</x:v>
       </x:c>
       <x:c r="F27" s="9" t="str">
-        <x:v>Do not select 0 or 1 yet. Application drafting can be parallel and repeatable, while formal review cycles are scarce and serial; the balance depends strongly on the licensing regime. Resolve together with the jurisdiction-specific licensing scope.</x:v>
+        <x:v>Do not select 0 or 1 yet. Licensing feedback speed is jurisdiction- and pathway-dependent, and the frozen row names no jurisdiction. A fusion-regulatory reviewer should determine whether a shared profile is defensible or whether U.S., Chinese and other licensing variants are required.</x:v>
       </x:c>
       <x:c r="G27" s="9" t="str">
-        <x:v>For that licensing regime, what counts as a formal attempt, what does it cost, and which parts of application preparation and substantive review can proceed in parallel?</x:v>
+        <x:v>Which jurisdiction-specific application, review and response stages define the ordinary fusion pilot licensing loop, and is any shared 0-1 recommendation defensible without a completed comparable case?</x:v>
       </x:c>
       <x:c r="H27" s="9" t="str">
-        <x:v>Preserve 0-1 pending a jurisdiction-specific attempt definition, respecting the unresolved owner disposition.</x:v>
+        <x:v>Carry 0-1 as an unadjudicated candidate range, not an empirical bound; do not select either owner-withheld value without a jurisdiction.</x:v>
       </x:c>
       <x:c r="I27" s="9" t="str">
         <x:v>fusion-src-039;fusion-src-040;fusion-src-004</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="76" customHeight="1">
+    <x:row r="28" ht="60" customHeight="1">
       <x:c r="A28" s="3" t="str">
         <x:v>sp-0030</x:v>
       </x:c>
       <x:c r="B28" s="3" t="str">
-        <x:v>S5</x:v>
+        <x:v>S3</x:v>
       </x:c>
       <x:c r="C28" s="3" t="str">
-        <x:v>0-2</x:v>
+        <x:v>0-1</x:v>
       </x:c>
       <x:c r="D28" s="3" t="str">
-        <x:v>requires_human_expert</x:v>
+        <x:v>requires_jurisdiction_variant</x:v>
       </x:c>
       <x:c r="E28" s="3" t="str">
-        <x:v>preserve_disagreement</x:v>
+        <x:v>needs_domain_review</x:v>
       </x:c>
       <x:c r="F28" s="3" t="str">
-        <x:v>Preserve the 0-2 disagreement pending the S5 clarification and regulatory domain review. An erroneous approval can have grave downstream consequences, so S5=2 is too permissive; however, harm also requires operation and additional conditions, so S5=0 is too absolute. A later adjudicated value may be 1, but it should not be manufactured from two model submissions.</x:v>
+        <x:v>Do not select 0 or 1 yet. Application drafting can be parallel and repeatable, while formal review cycles are scarce and serial; the balance depends strongly on the licensing regime. Resolve together with the jurisdiction-specific licensing scope.</x:v>
       </x:c>
       <x:c r="G28" s="3" t="str">
-        <x:v>What direct consequence can an erroneous fusion pilot licence or safety-case acceptance cause before the next genuinely independent operating authorization or technical control in that jurisdiction?</x:v>
+        <x:v>For that licensing regime, what counts as a formal attempt, what does it cost, and which parts of application preparation and substantive review can proceed in parallel?</x:v>
       </x:c>
       <x:c r="H28" s="3" t="str">
-        <x:v>Preserve the owner's 0-2 disagreement; do not manufacture 1 from two model marks.</x:v>
+        <x:v>Preserve 0-1 pending a jurisdiction-specific attempt definition, respecting the unresolved owner disposition.</x:v>
       </x:c>
       <x:c r="I28" s="3" t="str">
         <x:v>fusion-src-039;fusion-src-040;fusion-src-004</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="60" customHeight="1">
+    <x:row r="29" ht="76" customHeight="1">
       <x:c r="A29" s="9" t="str">
-        <x:v>sp-0031</x:v>
+        <x:v>sp-0030</x:v>
       </x:c>
       <x:c r="B29" s="9" t="str">
-        <x:v>S3</x:v>
+        <x:v>S5</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>0-1</x:v>
+        <x:v>0-2</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
-        <x:v>requires_pathway_variant</x:v>
+        <x:v>requires_human_expert</x:v>
       </x:c>
       <x:c r="E29" s="9" t="str">
-        <x:v>needs_better_evidence</x:v>
+        <x:v>preserve_disagreement</x:v>
       </x:c>
       <x:c r="F29" s="9" t="str">
-        <x:v>Preserve the 0-1 range. A pilot connection combines cheap study iterations with one scarce physical connection and energized test sequence. No directly comparable fusion-grid case exists, and site reuse, network strength and outage rules can change the topology.</x:v>
+        <x:v>Preserve the 0-2 disagreement pending the S5 clarification and regulatory domain review. An erroneous approval can have grave downstream consequences, so S5=2 is too permissive; however, harm also requires operation and additional conditions, so S5=0 is too absolute. A later adjudicated value may be 1, but it should not be manufactured from two model submissions.</x:v>
       </x:c>
       <x:c r="G29" s="9" t="str">
-        <x:v>For a concrete pilot site, which connection assets are reused or new, and what are the marginal cost and attainable repetition of studies versus energized integrated tests?</x:v>
+        <x:v>What direct consequence can an erroneous fusion pilot licence or safety-case acceptance cause before the next genuinely independent operating authorization or technical control in that jurisdiction?</x:v>
       </x:c>
       <x:c r="H29" s="9" t="str">
-        <x:v>Preserve the owner-requested 0-1 interval and route greenfield versus reused-site connection scope.</x:v>
+        <x:v>Preserve the owner's 0-2 disagreement; do not manufacture 1 from two model marks.</x:v>
       </x:c>
       <x:c r="I29" s="9" t="str">
-        <x:v>fusion-src-031</x:v>
+        <x:v>fusion-src-039;fusion-src-040;fusion-src-004</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="60" customHeight="1">
@@ -11398,7 +12296,7 @@
         <x:v>sp-0031</x:v>
       </x:c>
       <x:c r="B30" s="3" t="str">
-        <x:v>S4</x:v>
+        <x:v>S3</x:v>
       </x:c>
       <x:c r="C30" s="3" t="str">
         <x:v>0-1</x:v>
@@ -11410,44 +12308,73 @@
         <x:v>needs_better_evidence</x:v>
       </x:c>
       <x:c r="F30" s="3" t="str">
-        <x:v>Preserve the 0-1 range. Equipment delivery, switchyard work, outage windows and energization impose physical floors, but an existing power-plant site may reuse substantial infrastructure. The generic row is too underspecified for a single value without a site/pathway case.</x:v>
+        <x:v>Preserve the 0-1 range. A pilot connection combines cheap study iterations with one scarce physical connection and energized test sequence. No directly comparable fusion-grid case exists, and site reuse, network strength and outage rules can change the topology.</x:v>
       </x:c>
       <x:c r="G30" s="3" t="str">
-        <x:v>Which physical installation, connection and energization steps are unavoidable at that site, separately from equipment procurement queues, outage booking and regulatory waits?</x:v>
+        <x:v>For a concrete pilot site, which connection assets are reused or new, and what are the marginal cost and attainable repetition of studies versus energized integrated tests?</x:v>
       </x:c>
       <x:c r="H30" s="3" t="str">
-        <x:v>Preserve the owner 0-1 interval until the physical site/pathway topology is specified.</x:v>
+        <x:v>Preserve the owner-requested 0-1 interval and route greenfield versus reused-site connection scope.</x:v>
       </x:c>
       <x:c r="I30" s="3" t="str">
-        <x:v>missing</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="76" customHeight="1">
+        <x:v>fusion-src-031</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="60" customHeight="1">
       <x:c r="A31" s="9" t="str">
         <x:v>sp-0031</x:v>
       </x:c>
       <x:c r="B31" s="9" t="str">
+        <x:v>S4</x:v>
+      </x:c>
+      <x:c r="C31" s="9" t="str">
+        <x:v>0-1</x:v>
+      </x:c>
+      <x:c r="D31" s="9" t="str">
+        <x:v>requires_pathway_variant</x:v>
+      </x:c>
+      <x:c r="E31" s="9" t="str">
+        <x:v>needs_better_evidence</x:v>
+      </x:c>
+      <x:c r="F31" s="9" t="str">
+        <x:v>Preserve the 0-1 range. Equipment delivery, switchyard work, outage windows and energization impose physical floors, but an existing power-plant site may reuse substantial infrastructure. The generic row is too underspecified for a single value without a site/pathway case.</x:v>
+      </x:c>
+      <x:c r="G31" s="9" t="str">
+        <x:v>Which physical installation, connection and energization steps are unavoidable at that site, separately from equipment procurement queues, outage booking and regulatory waits?</x:v>
+      </x:c>
+      <x:c r="H31" s="9" t="str">
+        <x:v>Preserve the owner 0-1 interval until the physical site/pathway topology is specified.</x:v>
+      </x:c>
+      <x:c r="I31" s="9" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="76" customHeight="1">
+      <x:c r="A32" s="3" t="str">
+        <x:v>sp-0031</x:v>
+      </x:c>
+      <x:c r="B32" s="3" t="str">
         <x:v>S5</x:v>
       </x:c>
-      <x:c r="C31" s="9" t="str">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D31" s="9" t="str">
+      <x:c r="C32" s="3" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D32" s="3" t="str">
         <x:v>requires_human_expert</x:v>
       </x:c>
-      <x:c r="E31" s="9" t="str">
+      <x:c r="E32" s="3" t="str">
         <x:v>prefer_seed</x:v>
       </x:c>
-      <x:c r="F31" s="9" t="str">
+      <x:c r="F32" s="3" t="str">
         <x:v>Select S5=1. Protection or integration errors can damage equipment and disturb a shared network, but layered protection, staged energization and utility operating procedures normally limit the direct consequence. This is very low tolerance, not automatically catastrophic or irreversible.</x:v>
       </x:c>
-      <x:c r="G31" s="9" t="str">
+      <x:c r="G32" s="3" t="str">
         <x:v>What direct equipment or network consequences can incorrect pilot protection or energization cause before independently coordinated utility and plant protection isolate the fault?</x:v>
       </x:c>
-      <x:c r="H31" s="9" t="str">
+      <x:c r="H32" s="3" t="str">
         <x:v>Support owner 1 provisionally; the actual independent utility/plant boundary requires named review.</x:v>
       </x:c>
-      <x:c r="I31" s="9" t="str">
+      <x:c r="I32" s="3" t="str">
         <x:v>fusion-src-031</x:v>
       </x:c>
     </x:row>
@@ -11458,7 +12385,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b068e4665ab4266"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac83ac2347e9473d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11469,12 +12396,15 @@
   <x:cols>
     <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="11" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="115" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="97" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="75" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="115" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="97" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="75" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="23" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="37" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="54" customHeight="1">
@@ -11488,6 +12418,9 @@
       <x:c r="F1" s="5"/>
       <x:c r="G1" s="5"/>
       <x:c r="H1" s="5"/>
+      <x:c r="I1" s="5"/>
+      <x:c r="J1" s="5"/>
+      <x:c r="K1" s="5"/>
     </x:row>
     <x:row r="2" ht="43" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -11500,6 +12433,9 @@
       <x:c r="F2" s="6"/>
       <x:c r="G2" s="6"/>
       <x:c r="H2" s="6"/>
+      <x:c r="I2" s="6"/>
+      <x:c r="J2" s="6"/>
+      <x:c r="K2" s="6"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3"/>
@@ -11510,6 +12446,9 @@
       <x:c r="F3" s="3"/>
       <x:c r="G3" s="3"/>
       <x:c r="H3" s="3"/>
+      <x:c r="I3" s="3"/>
+      <x:c r="J3" s="3"/>
+      <x:c r="K3" s="3"/>
     </x:row>
     <x:row r="4" ht="43" customHeight="1">
       <x:c r="A4" s="8" t="str">
@@ -11519,21 +12458,30 @@
         <x:v>Dimension</x:v>
       </x:c>
       <x:c r="C4" s="8" t="str">
+        <x:v>Outreach package</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="str">
         <x:v>Question for named specialist</x:v>
       </x:c>
-      <x:c r="D4" s="8" t="str">
+      <x:c r="E4" s="8" t="str">
         <x:v>Why load-bearing</x:v>
       </x:c>
-      <x:c r="E4" s="8" t="str">
+      <x:c r="F4" s="8" t="str">
         <x:v>Canonical source IDs</x:v>
       </x:c>
-      <x:c r="F4" s="8" t="str">
+      <x:c r="G4" s="8" t="str">
         <x:v>Requested expertise</x:v>
       </x:c>
-      <x:c r="G4" s="8" t="str">
+      <x:c r="H4" s="8" t="str">
+        <x:v>Blocking stage</x:v>
+      </x:c>
+      <x:c r="I4" s="8" t="str">
+        <x:v>Draft-use status</x:v>
+      </x:c>
+      <x:c r="J4" s="8" t="str">
         <x:v>Named reviewer</x:v>
       </x:c>
-      <x:c r="H4" s="8" t="str">
+      <x:c r="K4" s="8" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
@@ -11545,21 +12493,30 @@
         <x:v>S2</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
+        <x:v>EXP-FUS-01</x:v>
+      </x:c>
+      <x:c r="D5" s="9" t="str">
         <x:v>For a representative pilot-relevant tokamak campaign, what is the ordinary selection-to-result-to-revision loop, and does the documented cadence support 1 or 2?</x:v>
       </x:c>
-      <x:c r="D5" s="9" t="str">
+      <x:c r="E5" s="9" t="str">
         <x:v>The owner prefers 1, but adjacent control papers do not resolve the elapsed selection feedback or the missing AI effect.</x:v>
       </x:c>
-      <x:c r="E5" s="9" t="str">
+      <x:c r="F5" s="9" t="str">
         <x:v>fusion-src-018;fusion-src-019;fusion-src-024</x:v>
       </x:c>
-      <x:c r="F5" s="9" t="str">
+      <x:c r="G5" s="9" t="str">
         <x:v>Named tokamak experimental programme or campaign scientist</x:v>
       </x:c>
-      <x:c r="G5" s="9" t="str">
+      <x:c r="H5" s="9" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I5" s="9" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J5" s="9" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H5" s="9" t="str">
+      <x:c r="K5" s="9" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11571,21 +12528,30 @@
         <x:v>S5</x:v>
       </x:c>
       <x:c r="C6" s="3" t="str">
+        <x:v>EXP-FUS-01</x:v>
+      </x:c>
+      <x:c r="D6" s="3" t="str">
         <x:v>At the pilot-relevant stored-energy and disruption envelope, what damage can an erroneous control output cause before independently verified machine protection acts?</x:v>
       </x:c>
-      <x:c r="D6" s="3" t="str">
+      <x:c r="E6" s="3" t="str">
         <x:v>Small-device proof of concept cannot establish the consequence boundary or support a universal 1.</x:v>
       </x:c>
-      <x:c r="E6" s="3" t="str">
+      <x:c r="F6" s="3" t="str">
         <x:v>fusion-src-018;fusion-src-008;fusion-src-020</x:v>
       </x:c>
-      <x:c r="F6" s="3" t="str">
+      <x:c r="G6" s="3" t="str">
         <x:v>Named tokamak plasma-control and machine-protection engineer</x:v>
       </x:c>
-      <x:c r="G6" s="3" t="str">
+      <x:c r="H6" s="3" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I6" s="3" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J6" s="3" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H6" s="3" t="str">
+      <x:c r="K6" s="3" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11597,21 +12563,30 @@
         <x:v>S3</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
+        <x:v>EXP-FUS-02</x:v>
+      </x:c>
+      <x:c r="D7" s="9" t="str">
         <x:v>Which material and pilot load envelope can the planned IFMIF-DONES specimen matrix represent, and how do spectrum/transmutation mismatch and accepted examinations limit useful parallel throughput?</x:v>
       </x:c>
-      <x:c r="D7" s="9" t="str">
+      <x:c r="E7" s="9" t="str">
         <x:v>Planned specimen capacity cannot be equated with accepted qualification throughput across materials.</x:v>
       </x:c>
-      <x:c r="E7" s="9" t="str">
+      <x:c r="F7" s="9" t="str">
         <x:v>fusion-src-045;fusion-src-046</x:v>
       </x:c>
-      <x:c r="F7" s="9" t="str">
+      <x:c r="G7" s="9" t="str">
         <x:v>Named fusion irradiation/materials-qualification specialist</x:v>
       </x:c>
-      <x:c r="G7" s="9" t="str">
+      <x:c r="H7" s="9" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I7" s="9" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J7" s="9" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H7" s="9" t="str">
+      <x:c r="K7" s="9" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11623,21 +12598,30 @@
         <x:v>S5</x:v>
       </x:c>
       <x:c r="C8" s="3" t="str">
+        <x:v>EXP-FUS-02</x:v>
+      </x:c>
+      <x:c r="D8" s="3" t="str">
         <x:v>Which losses from an invalid irradiation or examination programme are irreversible before independent component/material acceptance, and what qualification claims can escape that boundary?</x:v>
       </x:c>
-      <x:c r="D8" s="3" t="str">
+      <x:c r="E8" s="3" t="str">
         <x:v>The 0-1 disagreement depends on evidence loss and a real acceptance boundary, not a generic downstream accident.</x:v>
       </x:c>
-      <x:c r="E8" s="3" t="str">
+      <x:c r="F8" s="3" t="str">
         <x:v>fusion-src-045;fusion-src-046</x:v>
       </x:c>
-      <x:c r="F8" s="3" t="str">
+      <x:c r="G8" s="3" t="str">
         <x:v>Named fusion materials-qualification and assurance specialist</x:v>
       </x:c>
-      <x:c r="G8" s="3" t="str">
+      <x:c r="H8" s="3" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I8" s="3" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J8" s="3" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H8" s="3" t="str">
+      <x:c r="K8" s="3" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11649,21 +12633,30 @@
         <x:v>S4</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
+        <x:v>EXP-FUS-02</x:v>
+      </x:c>
+      <x:c r="D9" s="9" t="str">
         <x:v>Which neutron, heat-flux, thermal-cycling, erosion and maintainability exposures must occur inside the frozen PFC development stage, and can sequential tests represent their combined effects?</x:v>
       </x:c>
-      <x:c r="D9" s="9" t="str">
+      <x:c r="E9" s="9" t="str">
         <x:v>The evidence cannot establish whether the dominant physical floor warrants 0 or 1, and formal qualification must remain a separate stage.</x:v>
       </x:c>
-      <x:c r="E9" s="9" t="str">
+      <x:c r="F9" s="9" t="str">
         <x:v>fusion-src-026;fusion-src-045</x:v>
       </x:c>
-      <x:c r="F9" s="9" t="str">
+      <x:c r="G9" s="9" t="str">
         <x:v>Named plasma-facing component and plasma-material interaction specialist</x:v>
       </x:c>
-      <x:c r="G9" s="9" t="str">
+      <x:c r="H9" s="9" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I9" s="9" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J9" s="9" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H9" s="9" t="str">
+      <x:c r="K9" s="9" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11675,21 +12668,30 @@
         <x:v>S5</x:v>
       </x:c>
       <x:c r="C10" s="3" t="str">
+        <x:v>EXP-FUS-02</x:v>
+      </x:c>
+      <x:c r="D10" s="3" t="str">
         <x:v>What can an erroneous PFC development test or acceptance claim damage before the next independent acceptance/protection boundary, excluding failures discovered by a correctly conducted test?</x:v>
       </x:c>
-      <x:c r="D10" s="3" t="str">
+      <x:c r="E10" s="3" t="str">
         <x:v>This determines whether 1 or 2 is justified without charging later operational failures to development.</x:v>
       </x:c>
-      <x:c r="E10" s="3" t="str">
+      <x:c r="F10" s="3" t="str">
         <x:v>fusion-src-026</x:v>
       </x:c>
-      <x:c r="F10" s="3" t="str">
+      <x:c r="G10" s="3" t="str">
         <x:v>Named PFC test/qualification assurance engineer</x:v>
       </x:c>
-      <x:c r="G10" s="3" t="str">
+      <x:c r="H10" s="3" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I10" s="3" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J10" s="3" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H10" s="3" t="str">
+      <x:c r="K10" s="3" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11701,21 +12703,30 @@
         <x:v>S4</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
+        <x:v>EXP-FUS-03</x:v>
+      </x:c>
+      <x:c r="D11" s="9" t="str">
         <x:v>For the intended fuel-cycle subsystem tests, which retention, permeation, equilibration or residence processes impose irreducible duration, separately from authorization and facility-access delays?</x:v>
       </x:c>
-      <x:c r="D11" s="9" t="str">
+      <x:c r="E11" s="9" t="str">
         <x:v>Without this separation, institutional constraints are incorrectly counted as intrinsic S4 time floors.</x:v>
       </x:c>
-      <x:c r="E11" s="9" t="str">
+      <x:c r="F11" s="9" t="str">
         <x:v>fusion-src-038;fusion-src-028</x:v>
       </x:c>
-      <x:c r="F11" s="9" t="str">
+      <x:c r="G11" s="9" t="str">
         <x:v>Named tritium-processing and fuel-cycle engineer</x:v>
       </x:c>
-      <x:c r="G11" s="9" t="str">
+      <x:c r="H11" s="9" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I11" s="9" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J11" s="9" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H11" s="9" t="str">
+      <x:c r="K11" s="9" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11727,21 +12738,30 @@
         <x:v>S5</x:v>
       </x:c>
       <x:c r="C12" s="3" t="str">
+        <x:v>EXP-FUS-03</x:v>
+      </x:c>
+      <x:c r="D12" s="3" t="str">
         <x:v>What tritium inventory loss or release is reasonably foreseeable before independently verified secondary confinement and accountancy controls act in this development scope?</x:v>
       </x:c>
-      <x:c r="D12" s="3" t="str">
+      <x:c r="E12" s="3" t="str">
         <x:v>The owner preference of 1 cannot become an approved consequence judgment without a specific inventory and independent boundary.</x:v>
       </x:c>
-      <x:c r="E12" s="3" t="str">
+      <x:c r="F12" s="3" t="str">
         <x:v>fusion-src-038;fusion-src-028</x:v>
       </x:c>
-      <x:c r="F12" s="3" t="str">
+      <x:c r="G12" s="3" t="str">
         <x:v>Named tritium confinement, accountancy and radiological-safety specialist</x:v>
       </x:c>
-      <x:c r="G12" s="3" t="str">
+      <x:c r="H12" s="3" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I12" s="3" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J12" s="3" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H12" s="3" t="str">
+      <x:c r="K12" s="3" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11753,21 +12773,30 @@
         <x:v>S2</x:v>
       </x:c>
       <x:c r="C13" s="9" t="str">
+        <x:v>EXP-FUS-03</x:v>
+      </x:c>
+      <x:c r="D13" s="9" t="str">
         <x:v>For the specified blanket concept, does each decision-relevant development revision require integrated fusion-environment validation, or can representative subcomponent tests close an ordinary revision?</x:v>
       </x:c>
-      <x:c r="D13" s="9" t="str">
+      <x:c r="E13" s="9" t="str">
         <x:v>This tests the owner's 0 preference against the frozen development scope without calling future TBM operation completed qualification.</x:v>
       </x:c>
-      <x:c r="E13" s="9" t="str">
+      <x:c r="F13" s="9" t="str">
         <x:v>fusion-src-038;fusion-src-028</x:v>
       </x:c>
-      <x:c r="F13" s="9" t="str">
+      <x:c r="G13" s="9" t="str">
         <x:v>Named blanket systems and breeding-validation specialist</x:v>
       </x:c>
-      <x:c r="G13" s="9" t="str">
+      <x:c r="H13" s="9" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I13" s="9" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J13" s="9" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H13" s="9" t="str">
+      <x:c r="K13" s="9" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11779,21 +12808,30 @@
         <x:v>S5</x:v>
       </x:c>
       <x:c r="C14" s="3" t="str">
+        <x:v>EXP-FUS-03</x:v>
+      </x:c>
+      <x:c r="D14" s="3" t="str">
         <x:v>For that blanket concept, which erroneous development outputs can cause direct chemical, radiological or equipment harm before independent test isolation and integration acceptance?</x:v>
       </x:c>
-      <x:c r="D14" s="3" t="str">
+      <x:c r="E14" s="3" t="str">
         <x:v>Blanket concepts have different hazards, and neither generic catastrophic language nor complete containment is justified.</x:v>
       </x:c>
-      <x:c r="E14" s="3" t="str">
+      <x:c r="F14" s="3" t="str">
         <x:v>fusion-src-038;fusion-src-028</x:v>
       </x:c>
-      <x:c r="F14" s="3" t="str">
+      <x:c r="G14" s="3" t="str">
         <x:v>Named blanket engineering and test-safety specialist</x:v>
       </x:c>
-      <x:c r="G14" s="3" t="str">
+      <x:c r="H14" s="3" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I14" s="3" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J14" s="3" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H14" s="3" t="str">
+      <x:c r="K14" s="3" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11805,21 +12843,30 @@
         <x:v>S5</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
+        <x:v>EXP-FUS-04</x:v>
+      </x:c>
+      <x:c r="D15" s="9" t="str">
         <x:v>During pilot nuclear/tritium commissioning, what direct harm from an erroneous startup or interface check can occur before independently verified interlocks and readiness hold points act?</x:v>
       </x:c>
-      <x:c r="D15" s="9" t="str">
+      <x:c r="E15" s="9" t="str">
         <x:v>Low-power research-device first plasma does not validate the pilot boundary supporting owner 1.</x:v>
       </x:c>
-      <x:c r="E15" s="9" t="str">
+      <x:c r="F15" s="9" t="str">
         <x:v>fusion-src-033;fusion-src-034;fusion-src-036</x:v>
       </x:c>
-      <x:c r="F15" s="9" t="str">
+      <x:c r="G15" s="9" t="str">
         <x:v>Named fusion commissioning and nuclear/tritium systems-safety engineer</x:v>
       </x:c>
-      <x:c r="G15" s="9" t="str">
+      <x:c r="H15" s="9" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I15" s="9" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J15" s="9" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H15" s="9" t="str">
+      <x:c r="K15" s="9" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11831,21 +12878,30 @@
         <x:v>S2</x:v>
       </x:c>
       <x:c r="C16" s="3" t="str">
+        <x:v>EXP-FUS-04</x:v>
+      </x:c>
+      <x:c r="D16" s="3" t="str">
         <x:v>What specific pilot reliability or availability claim, exposure requirement and failure/repair criterion defines completion, and what ordinary learn-demonstrate-revise interval follows?</x:v>
       </x:c>
-      <x:c r="D16" s="3" t="str">
+      <x:c r="E16" s="3" t="str">
         <x:v>Pulse duration cannot establish a years-scale feedback claim, and the frozen profile does not name the reliability target.</x:v>
       </x:c>
-      <x:c r="E16" s="3" t="str">
+      <x:c r="F16" s="3" t="str">
         <x:v>fusion-src-011;fusion-src-032</x:v>
       </x:c>
-      <x:c r="F16" s="3" t="str">
+      <x:c r="G16" s="3" t="str">
         <x:v>Named fusion reliability/availability and maintainability specialist</x:v>
       </x:c>
-      <x:c r="G16" s="3" t="str">
+      <x:c r="H16" s="3" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I16" s="3" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J16" s="3" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H16" s="3" t="str">
+      <x:c r="K16" s="3" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11857,21 +12913,30 @@
         <x:v>S5</x:v>
       </x:c>
       <x:c r="C17" s="9" t="str">
+        <x:v>EXP-FUS-04</x:v>
+      </x:c>
+      <x:c r="D17" s="9" t="str">
         <x:v>Which errors in reliability-test conduct or inference can escape to cause harm before independent machine protection and readiness acceptance, distinct from component failures the test is meant to reveal?</x:v>
       </x:c>
-      <x:c r="D17" s="9" t="str">
+      <x:c r="E17" s="9" t="str">
         <x:v>This prevents both over-counting informative failures as catastrophic errors and understating false assurance.</x:v>
       </x:c>
-      <x:c r="E17" s="9" t="str">
+      <x:c r="F17" s="9" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="F17" s="9" t="str">
+      <x:c r="G17" s="9" t="str">
         <x:v>Named reliability demonstration and operational-assurance specialist</x:v>
       </x:c>
-      <x:c r="G17" s="9" t="str">
+      <x:c r="H17" s="9" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I17" s="9" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J17" s="9" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H17" s="9" t="str">
+      <x:c r="K17" s="9" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11883,21 +12948,30 @@
         <x:v>S2</x:v>
       </x:c>
       <x:c r="C18" s="3" t="str">
+        <x:v>EXP-FUS-05</x:v>
+      </x:c>
+      <x:c r="D18" s="3" t="str">
         <x:v>Which jurisdiction-specific application, review and response stages define the ordinary fusion pilot licensing loop, and is any shared 0-1 recommendation defensible without a completed comparable case?</x:v>
       </x:c>
-      <x:c r="D18" s="3" t="str">
+      <x:c r="E18" s="3" t="str">
         <x:v>The owner withheld selection; rulemaking intervals cannot resolve licensing feedback speed.</x:v>
       </x:c>
-      <x:c r="E18" s="3" t="str">
+      <x:c r="F18" s="3" t="str">
         <x:v>fusion-src-039;fusion-src-040;fusion-src-004</x:v>
       </x:c>
-      <x:c r="F18" s="3" t="str">
+      <x:c r="G18" s="3" t="str">
         <x:v>Named fusion regulatory specialist for the applicable jurisdiction; qualified Chinese legal reviewer for PRC wording</x:v>
       </x:c>
-      <x:c r="G18" s="3" t="str">
+      <x:c r="H18" s="3" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I18" s="3" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J18" s="3" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H18" s="3" t="str">
+      <x:c r="K18" s="3" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11909,21 +12983,30 @@
         <x:v>S3</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
+        <x:v>EXP-FUS-05</x:v>
+      </x:c>
+      <x:c r="D19" s="9" t="str">
         <x:v>For that licensing regime, what counts as a formal attempt, what does it cost, and which parts of application preparation and substantive review can proceed in parallel?</x:v>
       </x:c>
-      <x:c r="D19" s="9" t="str">
+      <x:c r="E19" s="9" t="str">
         <x:v>Cheap drafts and scarce formal reviews imply different S3 judgments; legal status supplies neither cost nor throughput.</x:v>
       </x:c>
-      <x:c r="E19" s="9" t="str">
+      <x:c r="F19" s="9" t="str">
         <x:v>fusion-src-039;fusion-src-040;fusion-src-004</x:v>
       </x:c>
-      <x:c r="F19" s="9" t="str">
+      <x:c r="G19" s="9" t="str">
         <x:v>Named fusion licensing practitioner with application and regulator-review experience</x:v>
       </x:c>
-      <x:c r="G19" s="9" t="str">
+      <x:c r="H19" s="9" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I19" s="9" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J19" s="9" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H19" s="9" t="str">
+      <x:c r="K19" s="9" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11935,21 +13018,30 @@
         <x:v>S5</x:v>
       </x:c>
       <x:c r="C20" s="3" t="str">
+        <x:v>EXP-FUS-05</x:v>
+      </x:c>
+      <x:c r="D20" s="3" t="str">
         <x:v>What direct consequence can an erroneous fusion pilot licence or safety-case acceptance cause before the next genuinely independent operating authorization or technical control in that jurisdiction?</x:v>
       </x:c>
-      <x:c r="D20" s="3" t="str">
+      <x:c r="E20" s="3" t="str">
         <x:v>The unresolved owner 0-2 interval depends on the actual legal and technical boundary; a midpoint would be fabricated consensus.</x:v>
       </x:c>
-      <x:c r="E20" s="3" t="str">
+      <x:c r="F20" s="3" t="str">
         <x:v>fusion-src-039;fusion-src-040;fusion-src-004</x:v>
       </x:c>
-      <x:c r="F20" s="3" t="str">
+      <x:c r="G20" s="3" t="str">
         <x:v>Named fusion regulatory/safety-case specialist; qualified native-language legal expertise where applicable</x:v>
       </x:c>
-      <x:c r="G20" s="3" t="str">
+      <x:c r="H20" s="3" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I20" s="3" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J20" s="3" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H20" s="3" t="str">
+      <x:c r="K20" s="3" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11961,21 +13053,30 @@
         <x:v>S3</x:v>
       </x:c>
       <x:c r="C21" s="9" t="str">
+        <x:v>EXP-FUS-06</x:v>
+      </x:c>
+      <x:c r="D21" s="9" t="str">
         <x:v>For a concrete pilot site, which connection assets are reused or new, and what are the marginal cost and attainable repetition of studies versus energized integrated tests?</x:v>
       </x:c>
-      <x:c r="D21" s="9" t="str">
+      <x:c r="E21" s="9" t="str">
         <x:v>The owner preserves 0-1 because no comparable fusion-grid case defines the decisive attempt set.</x:v>
       </x:c>
-      <x:c r="E21" s="9" t="str">
+      <x:c r="F21" s="9" t="str">
         <x:v>fusion-src-031</x:v>
       </x:c>
-      <x:c r="F21" s="9" t="str">
+      <x:c r="G21" s="9" t="str">
         <x:v>Named grid-interconnection and power-plant electrical engineer</x:v>
       </x:c>
-      <x:c r="G21" s="9" t="str">
+      <x:c r="H21" s="9" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I21" s="9" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J21" s="9" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H21" s="9" t="str">
+      <x:c r="K21" s="9" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -11987,21 +13088,30 @@
         <x:v>S4</x:v>
       </x:c>
       <x:c r="C22" s="3" t="str">
+        <x:v>EXP-FUS-06</x:v>
+      </x:c>
+      <x:c r="D22" s="3" t="str">
         <x:v>Which physical installation, connection and energization steps are unavoidable at that site, separately from equipment procurement queues, outage booking and regulatory waits?</x:v>
       </x:c>
-      <x:c r="D22" s="3" t="str">
+      <x:c r="E22" s="3" t="str">
         <x:v>Greenfield versus reused infrastructure can change the physical topology and the 0-1 recommendation.</x:v>
       </x:c>
-      <x:c r="E22" s="3" t="str">
+      <x:c r="F22" s="3" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="F22" s="3" t="str">
+      <x:c r="G22" s="3" t="str">
         <x:v>Named grid connection/construction and commissioning engineer</x:v>
       </x:c>
-      <x:c r="G22" s="3" t="str">
+      <x:c r="H22" s="3" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I22" s="3" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J22" s="3" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H22" s="3" t="str">
+      <x:c r="K22" s="3" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -12013,21 +13123,30 @@
         <x:v>S5</x:v>
       </x:c>
       <x:c r="C23" s="9" t="str">
+        <x:v>EXP-FUS-06</x:v>
+      </x:c>
+      <x:c r="D23" s="9" t="str">
         <x:v>What direct equipment or network consequences can incorrect pilot protection or energization cause before independently coordinated utility and plant protection isolate the fault?</x:v>
       </x:c>
-      <x:c r="D23" s="9" t="str">
+      <x:c r="E23" s="9" t="str">
         <x:v>Owner 1 depends on a real protection boundary that no observed fusion export case currently validates.</x:v>
       </x:c>
-      <x:c r="E23" s="9" t="str">
+      <x:c r="F23" s="9" t="str">
         <x:v>fusion-src-031</x:v>
       </x:c>
-      <x:c r="F23" s="9" t="str">
+      <x:c r="G23" s="9" t="str">
         <x:v>Named power-system protection and grid-integration safety engineer</x:v>
       </x:c>
-      <x:c r="G23" s="9" t="str">
+      <x:c r="H23" s="9" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="I23" s="9" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="J23" s="9" t="str">
         <x:v>missing</x:v>
       </x:c>
-      <x:c r="H23" s="9" t="str">
+      <x:c r="K23" s="9" t="str">
         <x:v>pending_named_specialist</x:v>
       </x:c>
     </x:row>
@@ -12038,12 +13157,254 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97891c01a6964ade"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f829761380348b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="55" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="78" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="37" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="100" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="54" customHeight="1">
+      <x:c r="A1" s="5" t="str">
+        <x:v>Outreach packages</x:v>
+      </x:c>
+      <x:c r="B1" s="5"/>
+      <x:c r="C1" s="5"/>
+      <x:c r="D1" s="5"/>
+      <x:c r="E1" s="5"/>
+      <x:c r="F1" s="5"/>
+      <x:c r="G1" s="5"/>
+      <x:c r="H1" s="5"/>
+    </x:row>
+    <x:row r="2" ht="43" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>AI-assisted · recommendation only. Details extend to the right.</x:v>
+      </x:c>
+      <x:c r="B2" s="6"/>
+      <x:c r="C2" s="6"/>
+      <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2" s="6"/>
+      <x:c r="H2" s="6"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="3"/>
+      <x:c r="B3" s="3"/>
+      <x:c r="C3" s="3"/>
+      <x:c r="D3" s="3"/>
+      <x:c r="E3" s="3"/>
+      <x:c r="F3" s="3"/>
+      <x:c r="G3" s="3"/>
+      <x:c r="H3" s="3"/>
+    </x:row>
+    <x:row r="4" ht="43" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>Package ID</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>Theme</x:v>
+      </x:c>
+      <x:c r="C4" s="8" t="str">
+        <x:v>Cell-level questions</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="str">
+        <x:v>Question count</x:v>
+      </x:c>
+      <x:c r="E4" s="8" t="str">
+        <x:v>Primary expertise</x:v>
+      </x:c>
+      <x:c r="F4" s="8" t="str">
+        <x:v>Blocking stage</x:v>
+      </x:c>
+      <x:c r="G4" s="8" t="str">
+        <x:v>Draft-use status</x:v>
+      </x:c>
+      <x:c r="H4" s="8" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="44" customHeight="1">
+      <x:c r="A5" s="9" t="str">
+        <x:v>EXP-FUS-01</x:v>
+      </x:c>
+      <x:c r="B5" s="9" t="str">
+        <x:v>Experiment campaigns, plasma control and machine protection</x:v>
+      </x:c>
+      <x:c r="C5" s="9" t="str">
+        <x:v>sp-0016/S2; sp-0018/S5</x:v>
+      </x:c>
+      <x:c r="D5" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E5" s="9" t="str">
+        <x:v>Tokamak campaign scientist; plasma-control and machine-protection engineer</x:v>
+      </x:c>
+      <x:c r="F5" s="9" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="G5" s="9" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="H5" s="9" t="str">
+        <x:v>Resolve experiment-selection cadence and the bounded machine-protection consequence boundary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="44" customHeight="1">
+      <x:c r="A6" s="3" t="str">
+        <x:v>EXP-FUS-02</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="str">
+        <x:v>Materials qualification and plasma-facing components</x:v>
+      </x:c>
+      <x:c r="C6" s="3" t="str">
+        <x:v>sp-0020/S3; sp-0020/S5; sp-0023/S4; sp-0023/S5</x:v>
+      </x:c>
+      <x:c r="D6" s="3" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E6" s="3" t="str">
+        <x:v>Fusion irradiation/materials-qualification and plasma-material-interaction specialists</x:v>
+      </x:c>
+      <x:c r="F6" s="3" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="G6" s="3" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="H6" s="3" t="str">
+        <x:v>Resolve representative throughput, irreversible evidence loss, combined-environment floors, and PFC assurance boundaries.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="44" customHeight="1">
+      <x:c r="A7" s="9" t="str">
+        <x:v>EXP-FUS-03</x:v>
+      </x:c>
+      <x:c r="B7" s="9" t="str">
+        <x:v>Tritium and blankets</x:v>
+      </x:c>
+      <x:c r="C7" s="9" t="str">
+        <x:v>sp-0024/S4; sp-0024/S5; sp-0025/S2; sp-0025/S5</x:v>
+      </x:c>
+      <x:c r="D7" s="9" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E7" s="9" t="str">
+        <x:v>Tritium processing/confinement and blanket engineering/test-safety specialists</x:v>
+      </x:c>
+      <x:c r="F7" s="9" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="G7" s="9" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="H7" s="9" t="str">
+        <x:v>Separate intrinsic process floors from access delays and define direct fuel-cycle/blanket consequences.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="44" customHeight="1">
+      <x:c r="A8" s="3" t="str">
+        <x:v>EXP-FUS-04</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="str">
+        <x:v>Commissioning and reliability</x:v>
+      </x:c>
+      <x:c r="C8" s="3" t="str">
+        <x:v>sp-0028/S5; sp-0029/S2; sp-0029/S5</x:v>
+      </x:c>
+      <x:c r="D8" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E8" s="3" t="str">
+        <x:v>Fusion commissioning, nuclear/tritium systems safety, reliability and maintainability specialists</x:v>
+      </x:c>
+      <x:c r="F8" s="3" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="G8" s="3" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="H8" s="3" t="str">
+        <x:v>Define pilot commissioning protection boundaries and the reliability claim/test protocol.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="44" customHeight="1">
+      <x:c r="A9" s="9" t="str">
+        <x:v>EXP-FUS-05</x:v>
+      </x:c>
+      <x:c r="B9" s="9" t="str">
+        <x:v>Licensing and regulation</x:v>
+      </x:c>
+      <x:c r="C9" s="9" t="str">
+        <x:v>sp-0030/S2; sp-0030/S3; sp-0030/S5</x:v>
+      </x:c>
+      <x:c r="D9" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E9" s="9" t="str">
+        <x:v>Fusion licensing practitioner/regulator; qualified Chinese legal reviewer for PRC wording</x:v>
+      </x:c>
+      <x:c r="F9" s="9" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="G9" s="9" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="H9" s="9" t="str">
+        <x:v>Define jurisdiction-specific review cycles, formal attempts, and the next genuinely independent authorization boundary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="44" customHeight="1">
+      <x:c r="A10" s="3" t="str">
+        <x:v>EXP-FUS-06</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="str">
+        <x:v>Grid integration and protection</x:v>
+      </x:c>
+      <x:c r="C10" s="3" t="str">
+        <x:v>sp-0031/S3; sp-0031/S4; sp-0031/S5</x:v>
+      </x:c>
+      <x:c r="D10" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E10" s="3" t="str">
+        <x:v>Grid-interconnection, power-plant electrical, construction/commissioning, and protection engineers</x:v>
+      </x:c>
+      <x:c r="F10" s="3" t="str">
+        <x:v>canonical_approval</x:v>
+      </x:c>
+      <x:c r="G10" s="3" t="str">
+        <x:v>allowed_as_expert_coded_draft</x:v>
+      </x:c>
+      <x:c r="H10" s="3" t="str">
+        <x:v>Resolve greenfield versus reused-site topology, physical connection floors, and the utility/plant protection boundary.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:D1"/>
+    <x:mergeCell ref="A2:D2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra12dafa029484cd6"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -15319,873 +16680,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c032d33a515483a"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="84" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="106" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="31" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="35" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="107" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="150" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="54" customHeight="1">
-      <x:c r="A1" s="5" t="str">
-        <x:v>Sources</x:v>
-      </x:c>
-      <x:c r="B1" s="5"/>
-      <x:c r="C1" s="5"/>
-      <x:c r="D1" s="5"/>
-      <x:c r="E1" s="5"/>
-      <x:c r="F1" s="5"/>
-      <x:c r="G1" s="5"/>
-      <x:c r="H1" s="5"/>
-    </x:row>
-    <x:row r="2" ht="43" customHeight="1">
-      <x:c r="A2" s="6" t="str">
-        <x:v>AI-assisted · recommendation only. Details extend to the right.</x:v>
-      </x:c>
-      <x:c r="B2" s="6"/>
-      <x:c r="C2" s="6"/>
-      <x:c r="D2" s="6"/>
-      <x:c r="E2" s="6"/>
-      <x:c r="F2" s="6"/>
-      <x:c r="G2" s="6"/>
-      <x:c r="H2" s="6"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="3"/>
-      <x:c r="B3" s="3"/>
-      <x:c r="C3" s="3"/>
-      <x:c r="D3" s="3"/>
-      <x:c r="E3" s="3"/>
-      <x:c r="F3" s="3"/>
-      <x:c r="G3" s="3"/>
-      <x:c r="H3" s="3"/>
-    </x:row>
-    <x:row r="4" ht="43" customHeight="1">
-      <x:c r="A4" s="8" t="str">
-        <x:v>Canonical source ID</x:v>
-      </x:c>
-      <x:c r="B4" s="8" t="str">
-        <x:v>Title</x:v>
-      </x:c>
-      <x:c r="C4" s="8" t="str">
-        <x:v>Primary / publisher URL</x:v>
-      </x:c>
-      <x:c r="D4" s="8" t="str">
-        <x:v>Independent-validation status</x:v>
-      </x:c>
-      <x:c r="E4" s="8" t="str">
-        <x:v>Evidence basis (bank)</x:v>
-      </x:c>
-      <x:c r="F4" s="8" t="str">
-        <x:v>Last verified</x:v>
-      </x:c>
-      <x:c r="G4" s="8" t="str">
-        <x:v>Source limitation</x:v>
-      </x:c>
-      <x:c r="H4" s="8" t="str">
-        <x:v>Promotion use restrictions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="76" customHeight="1">
-      <x:c r="A5" s="9" t="str">
-        <x:v>fusion-src-004</x:v>
-      </x:c>
-      <x:c r="B5" s="9" t="str">
-        <x:v>Atomic Energy Law of the People's Republic of China</x:v>
-      </x:c>
-      <x:c r="C5" s="9" t="str">
-        <x:v>https://www.caea.gov.cn/n6760338/n6760344/n10763762/n10763767/c10704020/content.html</x:v>
-      </x:c>
-      <x:c r="D5" s="9" t="str">
-        <x:v>not_applicable</x:v>
-      </x:c>
-      <x:c r="E5" s="9" t="str">
-        <x:v>observed legal/regulatory status</x:v>
-      </x:c>
-      <x:c r="F5" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G5" s="9" t="str">
-        <x:v>An enacted law establishes legal status and authority; it is not a completed fusion licensing case or evidence of review duration. Earlier draft numbering differed, and final Article 37 concerns disused radioactive-source recovery/disposal.</x:v>
-      </x:c>
-      <x:c r="H5" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. An enacted law establishes legal status and authority; it is not a completed fusion licensing case or evidence of review duration. Earlier draft numbering differed, and final Article 37 concerns disused radioactive-source recovery/disposal. Direct public quotation or load-bearing translated wording remains blocked until the stated native-language/specialist review is completed.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="44" customHeight="1">
-      <x:c r="A6" s="3" t="str">
-        <x:v>fusion-src-007</x:v>
-      </x:c>
-      <x:c r="B6" s="3" t="str">
-        <x:v>High-fidelity data-driven dynamics model for reinforcement learning-based control in HL-3 tokamak</x:v>
-      </x:c>
-      <x:c r="C6" s="3" t="str">
-        <x:v>https://doi.org/10.1038/s42005-025-02302-y</x:v>
-      </x:c>
-      <x:c r="D6" s="3" t="str">
-        <x:v>independently_validated</x:v>
-      </x:c>
-      <x:c r="E6" s="3" t="str">
-        <x:v>observed experimental result</x:v>
-      </x:c>
-      <x:c r="F6" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G6" s="3" t="str">
-        <x:v>Research-device demonstration; no nuclear-safety case, plant reliability, or transfer to pilot conditions.</x:v>
-      </x:c>
-      <x:c r="H6" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Research-device demonstration; no nuclear-safety case, plant reliability, or transfer to pilot conditions.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="44" customHeight="1">
-      <x:c r="A7" s="9" t="str">
-        <x:v>fusion-src-008</x:v>
-      </x:c>
-      <x:c r="B7" s="9" t="str">
-        <x:v>Interpretability analysis and real-time prediction of locked mode-induced disruptions in EAST</x:v>
-      </x:c>
-      <x:c r="C7" s="9" t="str">
-        <x:v>https://doi.org/10.1088/1361-6587/ade5c5</x:v>
-      </x:c>
-      <x:c r="D7" s="9" t="str">
-        <x:v>independently_validated</x:v>
-      </x:c>
-      <x:c r="E7" s="9" t="str">
-        <x:v>proof of concept</x:v>
-      </x:c>
-      <x:c r="F7" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G7" s="9" t="str">
-        <x:v>Prediction performance is not autonomous avoidance, safe termination, or pilot-plant error tolerance.</x:v>
-      </x:c>
-      <x:c r="H7" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Prediction performance is not autonomous avoidance, safe termination, or pilot-plant error tolerance.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="44" customHeight="1">
-      <x:c r="A8" s="3" t="str">
-        <x:v>fusion-src-009</x:v>
-      </x:c>
-      <x:c r="B8" s="3" t="str">
-        <x:v>Automatic identification of tokamak plasma confinement states with multi-task learning neural network</x:v>
-      </x:c>
-      <x:c r="C8" s="3" t="str">
-        <x:v>https://doi.org/10.1088/1741-4326/ade3ed</x:v>
-      </x:c>
-      <x:c r="D8" s="3" t="str">
-        <x:v>independently_validated</x:v>
-      </x:c>
-      <x:c r="E8" s="3" t="str">
-        <x:v>proof of concept</x:v>
-      </x:c>
-      <x:c r="F8" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G8" s="3" t="str">
-        <x:v>Classification benchmark; not a closed-loop control or safety demonstration.</x:v>
-      </x:c>
-      <x:c r="H8" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Classification benchmark; not a closed-loop control or safety demonstration.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="156" customHeight="1">
-      <x:c r="A9" s="9" t="str">
-        <x:v>fusion-src-011</x:v>
-      </x:c>
-      <x:c r="B9" s="9" t="str">
-        <x:v>Chinese fusion device sustains plasma operation for over 1,000 seconds</x:v>
-      </x:c>
-      <x:c r="C9" s="9" t="str">
-        <x:v>https://www.sh.news.cn/20260410/696d097c4a6c41b9af5f654314252a04/c.html</x:v>
-      </x:c>
-      <x:c r="D9" s="9" t="str">
-        <x:v>not_independently_validated</x:v>
-      </x:c>
-      <x:c r="E9" s="9" t="str">
-        <x:v>observed facility milestone</x:v>
-      </x:c>
-      <x:c r="F9" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G9" s="9" t="str">
-        <x:v>Official media repeats company data and explicitly describes low-parameter operation; not independent experimental validation, net energy, or plant availability.</x:v>
-      </x:c>
-      <x:c r="H9" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Official media repeats company data and explicitly describes low-parameter operation; not independent experimental validation, net energy, or plant availability. Reviewed source identity does not supply independent validation; company/operator reports and repeated company data must not be used as independently observed empirical outcomes. Rejected use fusion-rej-009: HH70 is a small, non-DT research tokamak without a breeder blanket, turbine, integrated tritium plant, or commercial nuclear commissioning. Permitted limited use: Optimistic analogue for small research-device iteration only. Do not transfer elapsed time to a pilot plant. Rejected use fusion-rej-010: Pulse duration and energy-turnover metrics omit blanket life, tritium-plant availability, component replacement, turbine/grid systems, downtime, and capacity factor. Permitted limited use: Plasma/facility milestone with device, discharge, and metric definitions preserved. No evidence of plant availability is implied.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="108" customHeight="1">
-      <x:c r="A10" s="3" t="str">
-        <x:v>fusion-src-012</x:v>
-      </x:c>
-      <x:c r="B10" s="3" t="str">
-        <x:v>HH70 achieves first plasma</x:v>
-      </x:c>
-      <x:c r="C10" s="3" t="str">
-        <x:v>https://energysingularity.cn/en/news/news-025.html</x:v>
-      </x:c>
-      <x:c r="D10" s="3" t="str">
-        <x:v>not_independently_validated</x:v>
-      </x:c>
-      <x:c r="E10" s="3" t="str">
-        <x:v>observed facility milestone</x:v>
-      </x:c>
-      <x:c r="F10" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G10" s="3" t="str">
-        <x:v>First-party milestone; small non-DT device without blanket, tritium plant, turbine, or commercial licensing.</x:v>
-      </x:c>
-      <x:c r="H10" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. First-party milestone; small non-DT device without blanket, tritium plant, turbine, or commercial licensing. Reviewed source identity does not supply independent validation; company/operator reports and repeated company data must not be used as independently observed empirical outcomes. Rejected use fusion-rej-009: HH70 is a small, non-DT research tokamak without a breeder blanket, turbine, integrated tritium plant, or commercial nuclear commissioning. Permitted limited use: Optimistic analogue for small research-device iteration only. Do not transfer elapsed time to a pilot plant.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="44" customHeight="1">
-      <x:c r="A11" s="9" t="str">
-        <x:v>fusion-src-014</x:v>
-      </x:c>
-      <x:c r="B11" s="9" t="str">
-        <x:v>Development and construction of magnet system for world's first full high temperature superconducting tokamak</x:v>
-      </x:c>
-      <x:c r="C11" s="9" t="str">
-        <x:v>https://doi.org/10.1016/j.supcon.2024.100137</x:v>
-      </x:c>
-      <x:c r="D11" s="9" t="str">
-        <x:v>independently_validated</x:v>
-      </x:c>
-      <x:c r="E11" s="9" t="str">
-        <x:v>proof of concept</x:v>
-      </x:c>
-      <x:c r="F11" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G11" s="9" t="str">
-        <x:v>Magnet engineering does not validate the 1,337-second AI causal claim or a fusion power plant.</x:v>
-      </x:c>
-      <x:c r="H11" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Magnet engineering does not validate the 1,337-second AI causal claim or a fusion power plant.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="44" customHeight="1">
-      <x:c r="A12" s="3" t="str">
-        <x:v>fusion-src-017</x:v>
-      </x:c>
-      <x:c r="B12" s="3" t="str">
-        <x:v>Magnetic control of tokamak plasmas through deep reinforcement learning</x:v>
-      </x:c>
-      <x:c r="C12" s="3" t="str">
-        <x:v>https://doi.org/10.1038/s41586-021-04301-9</x:v>
-      </x:c>
-      <x:c r="D12" s="3" t="str">
-        <x:v>independently_validated</x:v>
-      </x:c>
-      <x:c r="E12" s="3" t="str">
-        <x:v>observed experimental result</x:v>
-      </x:c>
-      <x:c r="F12" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G12" s="3" t="str">
-        <x:v>Research tokamak; does not establish pilot-plant transfer, safety, reliability, or reduced nuclear commissioning time.</x:v>
-      </x:c>
-      <x:c r="H12" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Research tokamak; does not establish pilot-plant transfer, safety, reliability, or reduced nuclear commissioning time.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="44" customHeight="1">
-      <x:c r="A13" s="9" t="str">
-        <x:v>fusion-src-018</x:v>
-      </x:c>
-      <x:c r="B13" s="9" t="str">
-        <x:v>Avoiding fusion plasma tearing instability with deep reinforcement learning</x:v>
-      </x:c>
-      <x:c r="C13" s="9" t="str">
-        <x:v>https://doi.org/10.1038/s41586-024-07024-9</x:v>
-      </x:c>
-      <x:c r="D13" s="9" t="str">
-        <x:v>independently_validated</x:v>
-      </x:c>
-      <x:c r="E13" s="9" t="str">
-        <x:v>observed experimental result</x:v>
-      </x:c>
-      <x:c r="F13" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G13" s="9" t="str">
-        <x:v>Early proof of concept on a research device; not universal disruption avoidance or a nuclear-safety system.</x:v>
-      </x:c>
-      <x:c r="H13" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Early proof of concept on a research device; not universal disruption avoidance or a nuclear-safety system.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="92" customHeight="1">
-      <x:c r="A14" s="3" t="str">
-        <x:v>fusion-src-019</x:v>
-      </x:c>
-      <x:c r="B14" s="3" t="str">
-        <x:v>Highest fusion performance without harmful edge energy bursts in tokamak</x:v>
-      </x:c>
-      <x:c r="C14" s="3" t="str">
-        <x:v>https://doi.org/10.1038/s41467-024-48415-w</x:v>
-      </x:c>
-      <x:c r="D14" s="3" t="str">
-        <x:v>independently_validated</x:v>
-      </x:c>
-      <x:c r="E14" s="3" t="str">
-        <x:v>observed experimental result</x:v>
-      </x:c>
-      <x:c r="F14" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G14" s="3" t="str">
-        <x:v>Device- and scenario-specific experiment; the pack's simplified 'up to 90%' line is not promoted without a metric-matched locator.</x:v>
-      </x:c>
-      <x:c r="H14" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Device- and scenario-specific experiment; the pack's simplified 'up to 90%' line is not promoted without a metric-matched locator. Rejected use fusion-rej-005: The paper reports several device- and metric-specific changes; the pack's compressed percentage omits the exact metric, denominator, device, and condition. Permitted limited use: Cite the peer-reviewed cross-device experiment qualitatively or extract a metric-specific value with a Results/figure locator. The source remains staged; only the simplified number is rejected.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="44" customHeight="1">
-      <x:c r="A15" s="9" t="str">
-        <x:v>fusion-src-020</x:v>
-      </x:c>
-      <x:c r="B15" s="9" t="str">
-        <x:v>Disruption prediction for future tokamaks using parameter-based transfer learning</x:v>
-      </x:c>
-      <x:c r="C15" s="9" t="str">
-        <x:v>https://doi.org/10.1038/s42005-023-01296-9</x:v>
-      </x:c>
-      <x:c r="D15" s="9" t="str">
-        <x:v>independently_validated</x:v>
-      </x:c>
-      <x:c r="E15" s="9" t="str">
-        <x:v>proof of concept</x:v>
-      </x:c>
-      <x:c r="F15" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G15" s="9" t="str">
-        <x:v>Offline, small-target-domain proof of concept; not live transfer to a future pilot plant.</x:v>
-      </x:c>
-      <x:c r="H15" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Offline, small-target-domain proof of concept; not live transfer to a future pilot plant.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="44" customHeight="1">
-      <x:c r="A16" s="3" t="str">
-        <x:v>fusion-src-021</x:v>
-      </x:c>
-      <x:c r="B16" s="3" t="str">
-        <x:v>Multimodal super-resolution: discovering hidden physics and its application to fusion plasmas</x:v>
-      </x:c>
-      <x:c r="C16" s="3" t="str">
-        <x:v>https://doi.org/10.1038/s41467-025-63492-1</x:v>
-      </x:c>
-      <x:c r="D16" s="3" t="str">
-        <x:v>independently_validated</x:v>
-      </x:c>
-      <x:c r="E16" s="3" t="str">
-        <x:v>proof of concept</x:v>
-      </x:c>
-      <x:c r="F16" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G16" s="3" t="str">
-        <x:v>Retrospective/synthetic diagnostic reconstruction; not a qualified replacement for safety instrumentation.</x:v>
-      </x:c>
-      <x:c r="H16" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Retrospective/synthetic diagnostic reconstruction; not a qualified replacement for safety instrumentation.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="44" customHeight="1">
-      <x:c r="A17" s="9" t="str">
-        <x:v>fusion-src-022</x:v>
-      </x:c>
-      <x:c r="B17" s="9" t="str">
-        <x:v>GS-DeepNet: mastering tokamak plasma equilibria with deep neural networks and the Grad–Shafranov equation</x:v>
-      </x:c>
-      <x:c r="C17" s="9" t="str">
-        <x:v>https://doi.org/10.1038/s41598-023-42991-5</x:v>
-      </x:c>
-      <x:c r="D17" s="9" t="str">
-        <x:v>independently_validated</x:v>
-      </x:c>
-      <x:c r="E17" s="9" t="str">
-        <x:v>proof of concept</x:v>
-      </x:c>
-      <x:c r="F17" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G17" s="9" t="str">
-        <x:v>Model benchmark; not a closed-loop or safety-qualified deployment.</x:v>
-      </x:c>
-      <x:c r="H17" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Model benchmark; not a closed-loop or safety-qualified deployment.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="60" customHeight="1">
-      <x:c r="A18" s="3" t="str">
-        <x:v>fusion-src-023</x:v>
-      </x:c>
-      <x:c r="B18" s="3" t="str">
-        <x:v>Finding the shadows in a fusion system faster with AI</x:v>
-      </x:c>
-      <x:c r="C18" s="3" t="str">
-        <x:v>https://www.pppl.gov/news/2025/finding-shadows-fusion-system-faster-ai</x:v>
-      </x:c>
-      <x:c r="D18" s="3" t="str">
-        <x:v>independently_validated</x:v>
-      </x:c>
-      <x:c r="E18" s="3" t="str">
-        <x:v>proof of concept</x:v>
-      </x:c>
-      <x:c r="F18" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G18" s="3" t="str">
-        <x:v>The present method covers 15 tiles in a small part of SPARC's exhaust geometry and is tied to that design; it is not plant-level schedule acceleration, materials qualification, or a generic plasma-facing-component result.</x:v>
-      </x:c>
-      <x:c r="H18" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. The present method covers 15 tiles in a small part of SPARC's exhaust geometry and is tied to that design; it is not plant-level schedule acceleration, materials qualification, or a generic plasma-facing-component result.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="60" customHeight="1">
-      <x:c r="A19" s="9" t="str">
-        <x:v>fusion-src-024</x:v>
-      </x:c>
-      <x:c r="B19" s="9" t="str">
-        <x:v>PPPL launches STELLAR-AI platform to accelerate fusion energy research</x:v>
-      </x:c>
-      <x:c r="C19" s="9" t="str">
-        <x:v>https://www.pppl.gov/news/2026/pppl-launches-stellar-ai-platform-accelerate-fusion-energy-research</x:v>
-      </x:c>
-      <x:c r="D19" s="9" t="str">
-        <x:v>not_applicable</x:v>
-      </x:c>
-      <x:c r="E19" s="9" t="str">
-        <x:v>programme announcement</x:v>
-      </x:c>
-      <x:c r="F19" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G19" s="9" t="str">
-        <x:v>Programme announcement and capability intent, not an observed AI-shortened research cycle; its 'NSTX-U this year' wording was superseded by a 2027 experiment target.</x:v>
-      </x:c>
-      <x:c r="H19" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Programme announcement and capability intent, not an observed AI-shortened research cycle; its 'NSTX-U this year' wording was superseded by a 2027 experiment target.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="92" customHeight="1">
-      <x:c r="A20" s="3" t="str">
-        <x:v>fusion-src-026</x:v>
-      </x:c>
-      <x:c r="B20" s="3" t="str">
-        <x:v>MPEX user research forum 2026</x:v>
-      </x:c>
-      <x:c r="C20" s="3" t="str">
-        <x:v>https://mpex.ornl.gov/murf-2026/</x:v>
-      </x:c>
-      <x:c r="D20" s="3" t="str">
-        <x:v>not_applicable</x:v>
-      </x:c>
-      <x:c r="E20" s="3" t="str">
-        <x:v>programme announcement</x:v>
-      </x:c>
-      <x:c r="F20" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G20" s="3" t="str">
-        <x:v>MPEX does not itself supply a fusion-spectrum neutron field; intended capability is not an observed qualification programme.</x:v>
-      </x:c>
-      <x:c r="H20" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. MPEX does not itself supply a fusion-spectrum neutron field; intended capability is not an observed qualification programme. Rejected use fusion-rej-011: MPEX is a plasma-materials exposure facility under assembly; it can test already neutron-irradiated specimens but is not itself a fusion-spectrum neutron source. Permitted limited use: Official intended capability for reactor-edge plasma exposure. Do not call intended capability completed qualification.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="44" customHeight="1">
-      <x:c r="A21" s="9" t="str">
-        <x:v>fusion-src-027</x:v>
-      </x:c>
-      <x:c r="B21" s="9" t="str">
-        <x:v>AI-accelerated fusion materials test facility</x:v>
-      </x:c>
-      <x:c r="C21" s="9" t="str">
-        <x:v>https://www.ornl.gov/research-highlight/ai-accelerated-fusion-materials-test-facility</x:v>
-      </x:c>
-      <x:c r="D21" s="9" t="str">
-        <x:v>not_applicable</x:v>
-      </x:c>
-      <x:c r="E21" s="9" t="str">
-        <x:v>programme announcement</x:v>
-      </x:c>
-      <x:c r="F21" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G21" s="9" t="str">
-        <x:v>Announced/developing capability, not demonstrated materials qualification or component-life acceleration.</x:v>
-      </x:c>
-      <x:c r="H21" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Announced/developing capability, not demonstrated materials qualification or component-life acceleration.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="44" customHeight="1">
-      <x:c r="A22" s="3" t="str">
-        <x:v>fusion-src-028</x:v>
-      </x:c>
-      <x:c r="B22" s="3" t="str">
-        <x:v>Fusion Science and Technology Roadmap</x:v>
-      </x:c>
-      <x:c r="C22" s="3" t="str">
-        <x:v>https://www.energy.gov/documents/fusion-science-and-technology-roadmap</x:v>
-      </x:c>
-      <x:c r="D22" s="3" t="str">
-        <x:v>not_applicable</x:v>
-      </x:c>
-      <x:c r="E22" s="3" t="str">
-        <x:v>programme announcement</x:v>
-      </x:c>
-      <x:c r="F22" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G22" s="3" t="str">
-        <x:v>Official roadmap and targets, not observed reductions in materials, blanket, tritium, licensing, or construction time.</x:v>
-      </x:c>
-      <x:c r="H22" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Official roadmap and targets, not observed reductions in materials, blanket, tritium, licensing, or construction time.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="60" customHeight="1">
-      <x:c r="A23" s="9" t="str">
-        <x:v>fusion-src-029</x:v>
-      </x:c>
-      <x:c r="B23" s="9" t="str">
-        <x:v>DIII-D National Fusion Program completes facility upgrade</x:v>
-      </x:c>
-      <x:c r="C23" s="9" t="str">
-        <x:v>https://www.ga.com/diii-d-national-fusion-program-completes-facility-upgrade</x:v>
-      </x:c>
-      <x:c r="D23" s="9" t="str">
-        <x:v>not_independently_validated</x:v>
-      </x:c>
-      <x:c r="E23" s="9" t="str">
-        <x:v>observed facility milestone</x:v>
-      </x:c>
-      <x:c r="F23" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G23" s="9" t="str">
-        <x:v>Facility milestone, not an AI result or a directly comparable nuclear commissioning programme.</x:v>
-      </x:c>
-      <x:c r="H23" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Facility milestone, not an AI result or a directly comparable nuclear commissioning programme. Reviewed source identity does not supply independent validation; company/operator reports and repeated company data must not be used as independently observed empirical outcomes.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="124" customHeight="1">
-      <x:c r="A24" s="3" t="str">
-        <x:v>fusion-src-031</x:v>
-      </x:c>
-      <x:c r="B24" s="3" t="str">
-        <x:v>SPARC technology page</x:v>
-      </x:c>
-      <x:c r="C24" s="3" t="str">
-        <x:v>https://www.cfs.energy/technology/</x:v>
-      </x:c>
-      <x:c r="D24" s="3" t="str">
-        <x:v>not_independently_validated</x:v>
-      </x:c>
-      <x:c r="E24" s="3" t="str">
-        <x:v>company target</x:v>
-      </x:c>
-      <x:c r="F24" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G24" s="3" t="str">
-        <x:v>Company target and living page; no observed Q&gt;1 result or grid connection.</x:v>
-      </x:c>
-      <x:c r="H24" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Company target and living page; no observed Q&gt;1 result or grid connection. Reviewed source identity does not supply independent validation; company/operator reports and repeated company data must not be used as independently observed empirical outcomes. Rejected use fusion-rej-013: Targets and programme announcements do not demonstrate net energy, electricity export, fuel self-sufficiency, availability, or grid connection. Permitted limited use: Target tracking with owner, date, pathway, and target status preserved. No target is typed as an observed result. Promotion freshness check 2026-09-01: CFS SPARC milestones still place construction in progress and first plasma/net energy in the future; no outcome approval.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="108" customHeight="1">
-      <x:c r="A25" s="9" t="str">
-        <x:v>fusion-src-032</x:v>
-      </x:c>
-      <x:c r="B25" s="9" t="str">
-        <x:v>New best values at Wendelstein 7-X</x:v>
-      </x:c>
-      <x:c r="C25" s="9" t="str">
-        <x:v>https://www.ipp.mpg.de/5532474/w7x</x:v>
-      </x:c>
-      <x:c r="D25" s="9" t="str">
-        <x:v>not_applicable</x:v>
-      </x:c>
-      <x:c r="E25" s="9" t="str">
-        <x:v>observed experimental result</x:v>
-      </x:c>
-      <x:c r="F25" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G25" s="9" t="str">
-        <x:v>Different discharges/metrics; neither is net energy, DT operation, plant availability, or blanket life.</x:v>
-      </x:c>
-      <x:c r="H25" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Different discharges/metrics; neither is net energy, DT operation, plant availability, or blanket life. Direct public quotation or load-bearing translated wording remains blocked until the stated native-language/specialist review is completed. Rejected use fusion-rej-010: Pulse duration and energy-turnover metrics omit blanket life, tritium-plant availability, component replacement, turbine/grid systems, downtime, and capacity factor. Permitted limited use: Plasma/facility milestone with device, discharge, and metric definitions preserved. No evidence of plant availability is implied.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="44" customHeight="1">
-      <x:c r="A26" s="3" t="str">
-        <x:v>fusion-src-033</x:v>
-      </x:c>
-      <x:c r="B26" s="3" t="str">
-        <x:v>First plasma 23 October</x:v>
-      </x:c>
-      <x:c r="C26" s="3" t="str">
-        <x:v>https://www.jt60sa.org/wp/first-plasma-23-october/</x:v>
-      </x:c>
-      <x:c r="D26" s="3" t="str">
-        <x:v>not_applicable</x:v>
-      </x:c>
-      <x:c r="E26" s="3" t="str">
-        <x:v>observed facility milestone</x:v>
-      </x:c>
-      <x:c r="F26" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G26" s="3" t="str">
-        <x:v>Low-power research commissioning milestone; not high-power operation, DT commissioning, or commercial reliability.</x:v>
-      </x:c>
-      <x:c r="H26" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Low-power research commissioning milestone; not high-power operation, DT commissioning, or commercial reliability.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="44" customHeight="1">
-      <x:c r="A27" s="9" t="str">
-        <x:v>fusion-src-034</x:v>
-      </x:c>
-      <x:c r="B27" s="9" t="str">
-        <x:v>OP2 has started</x:v>
-      </x:c>
-      <x:c r="C27" s="9" t="str">
-        <x:v>https://www.jt60sa.org/wp/op2-has-started/</x:v>
-      </x:c>
-      <x:c r="D27" s="9" t="str">
-        <x:v>not_applicable</x:v>
-      </x:c>
-      <x:c r="E27" s="9" t="str">
-        <x:v>official target</x:v>
-      </x:c>
-      <x:c r="F27" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G27" s="9" t="str">
-        <x:v>Mixed current facility milestone and future target; not proof that the experimental campaign or high-power commissioning is complete.</x:v>
-      </x:c>
-      <x:c r="H27" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Mixed current facility milestone and future target; not proof that the experimental campaign or high-power commissioning is complete.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="44" customHeight="1">
-      <x:c r="A28" s="3" t="str">
-        <x:v>fusion-src-036</x:v>
-      </x:c>
-      <x:c r="B28" s="3" t="str">
-        <x:v>ITER Machine Assembly Overview</x:v>
-      </x:c>
-      <x:c r="C28" s="3" t="str">
-        <x:v>https://www.iter.org/project/assembly-overview</x:v>
-      </x:c>
-      <x:c r="D28" s="3" t="str">
-        <x:v>not_applicable</x:v>
-      </x:c>
-      <x:c r="E28" s="3" t="str">
-        <x:v>official target</x:v>
-      </x:c>
-      <x:c r="F28" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G28" s="3" t="str">
-        <x:v>Official baseline proposal, not observed completion; later phases add nuclear/tritium systems.</x:v>
-      </x:c>
-      <x:c r="H28" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Official baseline proposal, not observed completion; later phases add nuclear/tritium systems.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="44" customHeight="1">
-      <x:c r="A29" s="9" t="str">
-        <x:v>fusion-src-037</x:v>
-      </x:c>
-      <x:c r="B29" s="9" t="str">
-        <x:v>Millions of data points, one successful lift</x:v>
-      </x:c>
-      <x:c r="C29" s="9" t="str">
-        <x:v>https://www.iter.org/node/20687/millions-data-points-one-successful-lift</x:v>
-      </x:c>
-      <x:c r="D29" s="9" t="str">
-        <x:v>not_applicable</x:v>
-      </x:c>
-      <x:c r="E29" s="9" t="str">
-        <x:v>observed facility milestone</x:v>
-      </x:c>
-      <x:c r="F29" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G29" s="9" t="str">
-        <x:v>Observed construction/facility milestone only; not an AI result, integrated chamber completion, commissioning, or plant completion.</x:v>
-      </x:c>
-      <x:c r="H29" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Observed construction/facility milestone only; not an AI result, integrated chamber completion, commissioning, or plant completion.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="44" customHeight="1">
-      <x:c r="A30" s="3" t="str">
-        <x:v>fusion-src-038</x:v>
-      </x:c>
-      <x:c r="B30" s="3" t="str">
-        <x:v>Tritium breeding</x:v>
-      </x:c>
-      <x:c r="C30" s="3" t="str">
-        <x:v>https://www.iter.org/machine/supporting-systems/tritium-breeding</x:v>
-      </x:c>
-      <x:c r="D30" s="3" t="str">
-        <x:v>not_applicable</x:v>
-      </x:c>
-      <x:c r="E30" s="3" t="str">
-        <x:v>programme announcement</x:v>
-      </x:c>
-      <x:c r="F30" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G30" s="3" t="str">
-        <x:v>Future test programme; ITER is not a tritium-self-sufficient power plant and testing is not qualification of a commercial blanket.</x:v>
-      </x:c>
-      <x:c r="H30" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Future test programme; ITER is not a tritium-self-sufficient power plant and testing is not qualification of a commercial blanket.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="44" customHeight="1">
-      <x:c r="A31" s="9" t="str">
-        <x:v>fusion-src-039</x:v>
-      </x:c>
-      <x:c r="B31" s="9" t="str">
-        <x:v>Regulatory Framework for Fusion Machines; Proposed Rule</x:v>
-      </x:c>
-      <x:c r="C31" s="9" t="str">
-        <x:v>https://www.federalregister.gov/documents/2026/02/26/2026-03865/regulatory-framework-for-fusion-machines</x:v>
-      </x:c>
-      <x:c r="D31" s="9" t="str">
-        <x:v>not_applicable</x:v>
-      </x:c>
-      <x:c r="E31" s="9" t="str">
-        <x:v>observed legal/regulatory status</x:v>
-      </x:c>
-      <x:c r="F31" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G31" s="9" t="str">
-        <x:v>Proposed rule and draft guidance, not a final rule, observed plant-licence review, or licence-review-duration dataset.</x:v>
-      </x:c>
-      <x:c r="H31" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Proposed rule and draft guidance, not a final rule, observed plant-licence review, or licence-review-duration dataset.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="76" customHeight="1">
-      <x:c r="A32" s="3" t="str">
-        <x:v>fusion-src-040</x:v>
-      </x:c>
-      <x:c r="B32" s="3" t="str">
-        <x:v>Fusion Machine Rulemaking Status</x:v>
-      </x:c>
-      <x:c r="C32" s="3" t="str">
-        <x:v>https://www.nrc.gov/materials/fusion/rulemaking-status</x:v>
-      </x:c>
-      <x:c r="D32" s="3" t="str">
-        <x:v>not_applicable</x:v>
-      </x:c>
-      <x:c r="E32" s="3" t="str">
-        <x:v>observed legal/regulatory status</x:v>
-      </x:c>
-      <x:c r="F32" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G32" s="3" t="str">
-        <x:v>Current regulator status, not evidence of licence throughput, a completed plant application, or licence-review duration.</x:v>
-      </x:c>
-      <x:c r="H32" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. Current regulator status, not evidence of licence throughput, a completed plant application, or licence-review duration. Promotion freshness check 2026-09-01: NRC status page still lists the February proposed rule and draft guidance; footer remains 2026-08-27. No final rule or completed licence case is inferred.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="60" customHeight="1">
-      <x:c r="A33" s="9" t="str">
-        <x:v>fusion-src-045</x:v>
-      </x:c>
-      <x:c r="B33" s="9" t="str">
-        <x:v>The IFMIF-DONES Irradiation Modules</x:v>
-      </x:c>
-      <x:c r="C33" s="9" t="str">
-        <x:v>https://doi.org/10.1088/1741-4326/add172</x:v>
-      </x:c>
-      <x:c r="D33" s="9" t="str">
-        <x:v>independently_validated</x:v>
-      </x:c>
-      <x:c r="E33" s="9" t="str">
-        <x:v>model or scenario estimate</x:v>
-      </x:c>
-      <x:c r="F33" s="9" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G33" s="9" t="str">
-        <x:v>IFMIF-DONES and its modules are under design/development; no completed or accepted qualification dataset exists. Spectrum/transmutation matching is material-dependent: Eurofer is tailored, while tungsten/copper conditions are not perfectly matched.</x:v>
-      </x:c>
-      <x:c r="H33" s="9" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. IFMIF-DONES and its modules are under design/development; no completed or accepted qualification dataset exists. Spectrum/transmutation matching is material-dependent: Eurofer is tailored, while tungsten/copper conditions are not perfectly matched.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="60" customHeight="1">
-      <x:c r="A34" s="3" t="str">
-        <x:v>fusion-src-046</x:v>
-      </x:c>
-      <x:c r="B34" s="3" t="str">
-        <x:v>IFMIF-DONES: Experimental strategy for fusion materials qualification</x:v>
-      </x:c>
-      <x:c r="C34" s="3" t="str">
-        <x:v>https://conferences.iaea.org/event/406/contributions/37622/</x:v>
-      </x:c>
-      <x:c r="D34" s="3" t="str">
-        <x:v>not_applicable</x:v>
-      </x:c>
-      <x:c r="E34" s="3" t="str">
-        <x:v>official target</x:v>
-      </x:c>
-      <x:c r="F34" s="3" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="G34" s="3" t="str">
-        <x:v>The facility is under construction and the values are programme design targets, not observed irradiation campaigns or a completed accepted qualification dataset. Post-irradiation examination remains part of the qualification chain.</x:v>
-      </x:c>
-      <x:c r="H34" s="3" t="str">
-        <x:v>Source-record review only; no claim approval, S-value selection, or profile approval. Fusion-domain review remains pending before profile use. The facility is under construction and the values are programme design targets, not observed irradiation campaigns or a completed accepted qualification dataset. Post-irradiation examination remains part of the qualification chain.</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:D1"/>
-    <x:mergeCell ref="A2:D2"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7519c5bc59404bbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4db1a378bfd4c07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>